<commit_message>
fuck the code im redoing the table
</commit_message>
<xml_diff>
--- a/static/data/Ratings.xlsx
+++ b/static/data/Ratings.xlsx
@@ -924,10 +924,13 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -939,13 +942,10 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1113,6 +1113,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFE4002C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF26F0CE"/>
         </patternFill>
       </fill>
@@ -1120,7 +1127,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF21976F"/>
+          <bgColor rgb="FFA8A8AB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1141,14 +1148,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDBDFE0"/>
+          <bgColor rgb="FF21976F"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFA8A8AB"/>
+          <bgColor rgb="FFDBDFE0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1177,13 +1184,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFD7F00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE4002C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2718,13 +2718,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:83" s="14" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
       <c r="F1" s="17"/>
       <c r="G1" s="17"/>
       <c r="H1" s="17"/>
@@ -2805,11 +2805,11 @@
       <c r="CE1" s="17"/>
     </row>
     <row r="2" spans="1:83" s="14" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
       <c r="F2" s="17"/>
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
@@ -2895,150 +2895,150 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
-      <c r="F3" s="39" t="e" vm="1">
+      <c r="F3" s="40" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G3" s="40"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="43" t="e" vm="2">
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="38" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="39" t="e" vm="3">
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="40" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O3" s="40"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="42" t="e" vm="4">
+      <c r="O3" s="41"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R3" s="43"/>
-      <c r="S3" s="43"/>
-      <c r="T3" s="43"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="42" t="e" vm="5">
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="38"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="37" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W3" s="43"/>
-      <c r="X3" s="43"/>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="39" t="e" vm="6">
+      <c r="W3" s="38"/>
+      <c r="X3" s="38"/>
+      <c r="Y3" s="38"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="40" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB3" s="40"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="39" t="e" vm="7">
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="42"/>
+      <c r="AD3" s="40" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE3" s="40"/>
-      <c r="AF3" s="41"/>
-      <c r="AG3" s="39" t="e" vm="8">
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="42"/>
+      <c r="AG3" s="40" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH3" s="40"/>
-      <c r="AI3" s="41"/>
-      <c r="AJ3" s="42" t="e" vm="9">
+      <c r="AH3" s="41"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="37" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK3" s="43"/>
-      <c r="AL3" s="43"/>
-      <c r="AM3" s="43"/>
-      <c r="AN3" s="44"/>
-      <c r="AO3" s="39" t="e" vm="10">
+      <c r="AK3" s="38"/>
+      <c r="AL3" s="38"/>
+      <c r="AM3" s="38"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="40" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP3" s="40"/>
-      <c r="AQ3" s="41"/>
-      <c r="AR3" s="39" t="e" vm="11">
+      <c r="AP3" s="41"/>
+      <c r="AQ3" s="42"/>
+      <c r="AR3" s="40" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS3" s="40"/>
-      <c r="AT3" s="41"/>
-      <c r="AU3" s="42" t="e" vm="12">
+      <c r="AS3" s="41"/>
+      <c r="AT3" s="42"/>
+      <c r="AU3" s="37" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV3" s="43"/>
-      <c r="AW3" s="43"/>
-      <c r="AX3" s="43"/>
-      <c r="AY3" s="44"/>
-      <c r="AZ3" s="39" t="e" vm="13">
+      <c r="AV3" s="38"/>
+      <c r="AW3" s="38"/>
+      <c r="AX3" s="38"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="40" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA3" s="40"/>
-      <c r="BB3" s="41"/>
-      <c r="BC3" s="39" t="e" vm="7">
+      <c r="BA3" s="41"/>
+      <c r="BB3" s="42"/>
+      <c r="BC3" s="40" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD3" s="40"/>
-      <c r="BE3" s="41"/>
-      <c r="BF3" s="39" t="e" vm="14">
+      <c r="BD3" s="41"/>
+      <c r="BE3" s="42"/>
+      <c r="BF3" s="40" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG3" s="40"/>
-      <c r="BH3" s="41"/>
-      <c r="BI3" s="42" t="e" vm="15">
+      <c r="BG3" s="41"/>
+      <c r="BH3" s="42"/>
+      <c r="BI3" s="37" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ3" s="43"/>
-      <c r="BK3" s="43"/>
-      <c r="BL3" s="43"/>
-      <c r="BM3" s="44"/>
-      <c r="BN3" s="39" t="e" vm="4">
+      <c r="BJ3" s="38"/>
+      <c r="BK3" s="38"/>
+      <c r="BL3" s="38"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="40" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO3" s="40"/>
-      <c r="BP3" s="41"/>
-      <c r="BQ3" s="39" t="e" vm="16">
+      <c r="BO3" s="41"/>
+      <c r="BP3" s="42"/>
+      <c r="BQ3" s="40" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR3" s="40"/>
-      <c r="BS3" s="41"/>
-      <c r="BT3" s="39" t="e" vm="17">
+      <c r="BR3" s="41"/>
+      <c r="BS3" s="42"/>
+      <c r="BT3" s="40" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU3" s="40"/>
-      <c r="BV3" s="41"/>
-      <c r="BW3" s="39" t="e" vm="4">
+      <c r="BU3" s="41"/>
+      <c r="BV3" s="42"/>
+      <c r="BW3" s="40" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX3" s="40"/>
-      <c r="BY3" s="41"/>
-      <c r="BZ3" s="39" t="e" vm="18">
+      <c r="BX3" s="41"/>
+      <c r="BY3" s="42"/>
+      <c r="BZ3" s="40" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA3" s="40"/>
-      <c r="CB3" s="41"/>
-      <c r="CC3" s="39" t="e" vm="19">
+      <c r="CA3" s="41"/>
+      <c r="CB3" s="42"/>
+      <c r="CC3" s="40" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD3" s="40"/>
-      <c r="CE3" s="41"/>
+      <c r="CD3" s="41"/>
+      <c r="CE3" s="42"/>
     </row>
     <row r="4" spans="1:83" s="16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="32" t="s">
@@ -9458,150 +9458,150 @@
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
-      <c r="F29" s="42" t="e" vm="1">
+      <c r="F29" s="37" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="43" t="e" vm="2">
+      <c r="G29" s="38"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="38" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J29" s="43"/>
-      <c r="K29" s="43"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="42" t="e" vm="3">
+      <c r="J29" s="38"/>
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="37" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O29" s="43"/>
-      <c r="P29" s="44"/>
-      <c r="Q29" s="43" t="e" vm="4">
+      <c r="O29" s="38"/>
+      <c r="P29" s="39"/>
+      <c r="Q29" s="38" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R29" s="43"/>
-      <c r="S29" s="43"/>
-      <c r="T29" s="43"/>
-      <c r="U29" s="44"/>
-      <c r="V29" s="42" t="e" vm="5">
+      <c r="R29" s="38"/>
+      <c r="S29" s="38"/>
+      <c r="T29" s="38"/>
+      <c r="U29" s="39"/>
+      <c r="V29" s="37" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W29" s="43"/>
-      <c r="X29" s="43"/>
-      <c r="Y29" s="43"/>
-      <c r="Z29" s="43"/>
-      <c r="AA29" s="42" t="e" vm="6">
+      <c r="W29" s="38"/>
+      <c r="X29" s="38"/>
+      <c r="Y29" s="38"/>
+      <c r="Z29" s="38"/>
+      <c r="AA29" s="37" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB29" s="43"/>
-      <c r="AC29" s="44"/>
-      <c r="AD29" s="42" t="e" vm="7">
+      <c r="AB29" s="38"/>
+      <c r="AC29" s="39"/>
+      <c r="AD29" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE29" s="43"/>
-      <c r="AF29" s="44"/>
-      <c r="AG29" s="42" t="e" vm="8">
+      <c r="AE29" s="38"/>
+      <c r="AF29" s="39"/>
+      <c r="AG29" s="37" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH29" s="43"/>
-      <c r="AI29" s="44"/>
-      <c r="AJ29" s="43" t="e" vm="9">
+      <c r="AH29" s="38"/>
+      <c r="AI29" s="39"/>
+      <c r="AJ29" s="38" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK29" s="43"/>
-      <c r="AL29" s="43"/>
-      <c r="AM29" s="43"/>
-      <c r="AN29" s="43"/>
-      <c r="AO29" s="42" t="e" vm="10">
+      <c r="AK29" s="38"/>
+      <c r="AL29" s="38"/>
+      <c r="AM29" s="38"/>
+      <c r="AN29" s="38"/>
+      <c r="AO29" s="37" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP29" s="43"/>
-      <c r="AQ29" s="44"/>
-      <c r="AR29" s="42" t="e" vm="11">
+      <c r="AP29" s="38"/>
+      <c r="AQ29" s="39"/>
+      <c r="AR29" s="37" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS29" s="43"/>
-      <c r="AT29" s="44"/>
-      <c r="AU29" s="43" t="e" vm="12">
+      <c r="AS29" s="38"/>
+      <c r="AT29" s="39"/>
+      <c r="AU29" s="38" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV29" s="43"/>
-      <c r="AW29" s="43"/>
-      <c r="AX29" s="43"/>
-      <c r="AY29" s="43"/>
-      <c r="AZ29" s="42" t="e" vm="13">
+      <c r="AV29" s="38"/>
+      <c r="AW29" s="38"/>
+      <c r="AX29" s="38"/>
+      <c r="AY29" s="38"/>
+      <c r="AZ29" s="37" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA29" s="43"/>
-      <c r="BB29" s="44"/>
-      <c r="BC29" s="42" t="e" vm="7">
+      <c r="BA29" s="38"/>
+      <c r="BB29" s="39"/>
+      <c r="BC29" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD29" s="43"/>
-      <c r="BE29" s="44"/>
-      <c r="BF29" s="42" t="e" vm="14">
+      <c r="BD29" s="38"/>
+      <c r="BE29" s="39"/>
+      <c r="BF29" s="37" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG29" s="43"/>
-      <c r="BH29" s="44"/>
-      <c r="BI29" s="43" t="e" vm="15">
+      <c r="BG29" s="38"/>
+      <c r="BH29" s="39"/>
+      <c r="BI29" s="38" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ29" s="43"/>
-      <c r="BK29" s="43"/>
-      <c r="BL29" s="43"/>
-      <c r="BM29" s="43"/>
-      <c r="BN29" s="42" t="e" vm="4">
+      <c r="BJ29" s="38"/>
+      <c r="BK29" s="38"/>
+      <c r="BL29" s="38"/>
+      <c r="BM29" s="38"/>
+      <c r="BN29" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO29" s="43"/>
-      <c r="BP29" s="44"/>
-      <c r="BQ29" s="42" t="e" vm="16">
+      <c r="BO29" s="38"/>
+      <c r="BP29" s="39"/>
+      <c r="BQ29" s="37" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR29" s="43"/>
-      <c r="BS29" s="44"/>
-      <c r="BT29" s="42" t="e" vm="17">
+      <c r="BR29" s="38"/>
+      <c r="BS29" s="39"/>
+      <c r="BT29" s="37" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU29" s="43"/>
-      <c r="BV29" s="44"/>
-      <c r="BW29" s="42" t="e" vm="4">
+      <c r="BU29" s="38"/>
+      <c r="BV29" s="39"/>
+      <c r="BW29" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX29" s="43"/>
-      <c r="BY29" s="44"/>
-      <c r="BZ29" s="42" t="e" vm="18">
+      <c r="BX29" s="38"/>
+      <c r="BY29" s="39"/>
+      <c r="BZ29" s="37" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA29" s="43"/>
-      <c r="CB29" s="44"/>
-      <c r="CC29" s="42" t="e" vm="19">
+      <c r="CA29" s="38"/>
+      <c r="CB29" s="39"/>
+      <c r="CC29" s="37" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD29" s="43"/>
-      <c r="CE29" s="44"/>
+      <c r="CD29" s="38"/>
+      <c r="CE29" s="39"/>
     </row>
     <row r="30" spans="1:83" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="32" t="s">
@@ -15532,18 +15532,67 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="I30:M30"/>
-    <mergeCell ref="N30:P30"/>
-    <mergeCell ref="BW30:BY30"/>
-    <mergeCell ref="BZ30:CB30"/>
-    <mergeCell ref="CC30:CE30"/>
-    <mergeCell ref="AZ30:BB30"/>
-    <mergeCell ref="BC30:BE30"/>
-    <mergeCell ref="BF30:BH30"/>
-    <mergeCell ref="BI30:BM30"/>
-    <mergeCell ref="BN30:BP30"/>
-    <mergeCell ref="BQ30:BS30"/>
+    <mergeCell ref="AA4:AC4"/>
+    <mergeCell ref="AD4:AF4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="AJ4:AN4"/>
+    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="Q3:U3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="AR29:AT29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="N29:P29"/>
+    <mergeCell ref="Q29:U29"/>
+    <mergeCell ref="V29:Z29"/>
+    <mergeCell ref="V4:Z4"/>
+    <mergeCell ref="AG3:AI3"/>
+    <mergeCell ref="AJ3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="BW3:BY3"/>
+    <mergeCell ref="BZ3:CB3"/>
+    <mergeCell ref="CC3:CE3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="V3:Z3"/>
+    <mergeCell ref="AA3:AC3"/>
+    <mergeCell ref="AD3:AF3"/>
+    <mergeCell ref="BT3:BV3"/>
+    <mergeCell ref="AU3:AY3"/>
+    <mergeCell ref="AZ3:BB3"/>
+    <mergeCell ref="BC3:BE3"/>
+    <mergeCell ref="BF3:BH3"/>
+    <mergeCell ref="BI3:BM3"/>
+    <mergeCell ref="BN3:BP3"/>
+    <mergeCell ref="BQ3:BS3"/>
+    <mergeCell ref="CC4:CE4"/>
+    <mergeCell ref="AR4:AT4"/>
+    <mergeCell ref="AU4:AY4"/>
+    <mergeCell ref="AZ4:BB4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="BF4:BH4"/>
+    <mergeCell ref="BI4:BM4"/>
+    <mergeCell ref="BN4:BP4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BT4:BV4"/>
+    <mergeCell ref="BW4:BY4"/>
+    <mergeCell ref="BZ4:CB4"/>
+    <mergeCell ref="BQ29:BS29"/>
+    <mergeCell ref="BT29:BV29"/>
+    <mergeCell ref="AG29:AI29"/>
+    <mergeCell ref="AJ29:AN29"/>
+    <mergeCell ref="AO29:AQ29"/>
     <mergeCell ref="BW29:BY29"/>
     <mergeCell ref="BZ29:CB29"/>
     <mergeCell ref="CC29:CE29"/>
@@ -15560,77 +15609,28 @@
     <mergeCell ref="BN29:BP29"/>
     <mergeCell ref="AA29:AC29"/>
     <mergeCell ref="AD29:AF29"/>
+    <mergeCell ref="CC30:CE30"/>
+    <mergeCell ref="AZ30:BB30"/>
+    <mergeCell ref="BC30:BE30"/>
+    <mergeCell ref="BF30:BH30"/>
+    <mergeCell ref="BI30:BM30"/>
+    <mergeCell ref="BN30:BP30"/>
+    <mergeCell ref="BQ30:BS30"/>
+    <mergeCell ref="BT30:BV30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:M30"/>
+    <mergeCell ref="N30:P30"/>
+    <mergeCell ref="BW30:BY30"/>
+    <mergeCell ref="BZ30:CB30"/>
     <mergeCell ref="Q30:U30"/>
     <mergeCell ref="V30:Z30"/>
     <mergeCell ref="AA30:AC30"/>
-    <mergeCell ref="BQ29:BS29"/>
-    <mergeCell ref="BT29:BV29"/>
-    <mergeCell ref="AG29:AI29"/>
-    <mergeCell ref="AJ29:AN29"/>
-    <mergeCell ref="AO29:AQ29"/>
-    <mergeCell ref="BT30:BV30"/>
     <mergeCell ref="AD30:AF30"/>
     <mergeCell ref="AG30:AI30"/>
     <mergeCell ref="AJ30:AN30"/>
     <mergeCell ref="AO30:AQ30"/>
     <mergeCell ref="AR30:AT30"/>
     <mergeCell ref="AU30:AY30"/>
-    <mergeCell ref="CC4:CE4"/>
-    <mergeCell ref="AR4:AT4"/>
-    <mergeCell ref="AU4:AY4"/>
-    <mergeCell ref="AZ4:BB4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="BF4:BH4"/>
-    <mergeCell ref="BI4:BM4"/>
-    <mergeCell ref="BN4:BP4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BT4:BV4"/>
-    <mergeCell ref="BW4:BY4"/>
-    <mergeCell ref="BZ4:CB4"/>
-    <mergeCell ref="BW3:BY3"/>
-    <mergeCell ref="BZ3:CB3"/>
-    <mergeCell ref="CC3:CE3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="V3:Z3"/>
-    <mergeCell ref="AA3:AC3"/>
-    <mergeCell ref="AD3:AF3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="AR29:AT29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="N29:P29"/>
-    <mergeCell ref="Q29:U29"/>
-    <mergeCell ref="V29:Z29"/>
-    <mergeCell ref="V4:Z4"/>
-    <mergeCell ref="BT3:BV3"/>
-    <mergeCell ref="AG3:AI3"/>
-    <mergeCell ref="AJ3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="AU3:AY3"/>
-    <mergeCell ref="AZ3:BB3"/>
-    <mergeCell ref="BC3:BE3"/>
-    <mergeCell ref="BF3:BH3"/>
-    <mergeCell ref="BI3:BM3"/>
-    <mergeCell ref="BN3:BP3"/>
-    <mergeCell ref="BQ3:BS3"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="Q3:U3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="AA4:AC4"/>
-    <mergeCell ref="AD4:AF4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="AJ4:AN4"/>
-    <mergeCell ref="AO4:AQ4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B27 D6:D27 B32:B53 D32:D53">
     <cfRule type="expression" dxfId="65" priority="329">
@@ -16684,7 +16684,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2 G4 G6 G8 G10 G12 G14 G16 G18 G20 G22">
+  <conditionalFormatting sqref="G4 G2 G6 G8 G10 G12 G14 G16 G18 G20 G22">
     <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="percentile" val="0"/>
@@ -16744,38 +16744,38 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2 O2 H2:H3 J2:J3">
-    <cfRule type="expression" dxfId="32" priority="347">
-      <formula>$J2="Ferrari"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="31" priority="348">
+    <cfRule type="expression" dxfId="32" priority="348">
       <formula>$J2="McLaren"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="349">
+    <cfRule type="expression" dxfId="31" priority="349">
       <formula>$J2="Red Bull"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="350">
+    <cfRule type="expression" dxfId="30" priority="350">
       <formula>$J2="Alpine"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="351">
+    <cfRule type="expression" dxfId="29" priority="351">
       <formula>$J2="Racing Bulls"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="344">
+    <cfRule type="expression" dxfId="28" priority="352">
+      <formula>$J2="Haas"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="345">
+      <formula>$J2="Aston Martin"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="342">
+      <formula>$J2="Williams"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="343">
+      <formula>$J2="Audi"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="344">
       <formula>$J2="Cadillac"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="352">
-      <formula>$J2="Haas"</formula>
+    <cfRule type="expression" dxfId="23" priority="346">
+      <formula>$J2="Mercedes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="342">
-      <formula>$J2="Williams"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="343">
-      <formula>$J2="Audi"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="23" priority="345">
-      <formula>$J2="Aston Martin"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="346">
-      <formula>$J2="Mercedes"</formula>
+    <cfRule type="expression" dxfId="22" priority="347">
+      <formula>$J2="Ferrari"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M12">

</xml_diff>

<commit_message>
lec ham rating swap fixed
</commit_message>
<xml_diff>
--- a/static/data/Ratings.xlsx
+++ b/static/data/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Programming\webdev\portfolio\static\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC51BD6-B6D8-45CB-8B07-1C39270728F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB68969A-3BD9-4485-8BE5-55D3B8DFED46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="2" activeTab="2" xr2:uid="{BD88BCC4-2E11-4C36-830D-A75A044EF5A6}"/>
   </bookViews>
@@ -924,12 +924,6 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -946,6 +940,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2718,13 +2718,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:83" s="14" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
       <c r="F1" s="17"/>
       <c r="G1" s="17"/>
       <c r="H1" s="17"/>
@@ -2805,11 +2805,11 @@
       <c r="CE1" s="17"/>
     </row>
     <row r="2" spans="1:83" s="14" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
       <c r="F2" s="17"/>
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
@@ -2895,150 +2895,150 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
-      <c r="F3" s="42" t="e" vm="1">
+      <c r="F3" s="40" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="40" t="e" vm="2">
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="38" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="42" t="e" vm="3">
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="40" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O3" s="43"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="39" t="e" vm="4">
+      <c r="O3" s="41"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="41"/>
-      <c r="V3" s="39" t="e" vm="5">
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="38"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="37" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W3" s="40"/>
-      <c r="X3" s="40"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="41"/>
-      <c r="AA3" s="42" t="e" vm="6">
+      <c r="W3" s="38"/>
+      <c r="X3" s="38"/>
+      <c r="Y3" s="38"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="40" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB3" s="43"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="42" t="e" vm="7">
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="42"/>
+      <c r="AD3" s="40" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="42" t="e" vm="8">
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="42"/>
+      <c r="AG3" s="40" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH3" s="43"/>
-      <c r="AI3" s="44"/>
-      <c r="AJ3" s="39" t="e" vm="9">
+      <c r="AH3" s="41"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="37" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK3" s="40"/>
-      <c r="AL3" s="40"/>
-      <c r="AM3" s="40"/>
-      <c r="AN3" s="41"/>
-      <c r="AO3" s="42" t="e" vm="10">
+      <c r="AK3" s="38"/>
+      <c r="AL3" s="38"/>
+      <c r="AM3" s="38"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="40" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP3" s="43"/>
-      <c r="AQ3" s="44"/>
-      <c r="AR3" s="42" t="e" vm="11">
+      <c r="AP3" s="41"/>
+      <c r="AQ3" s="42"/>
+      <c r="AR3" s="40" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS3" s="43"/>
-      <c r="AT3" s="44"/>
-      <c r="AU3" s="39" t="e" vm="12">
+      <c r="AS3" s="41"/>
+      <c r="AT3" s="42"/>
+      <c r="AU3" s="37" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV3" s="40"/>
-      <c r="AW3" s="40"/>
-      <c r="AX3" s="40"/>
-      <c r="AY3" s="41"/>
-      <c r="AZ3" s="42" t="e" vm="13">
+      <c r="AV3" s="38"/>
+      <c r="AW3" s="38"/>
+      <c r="AX3" s="38"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="40" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA3" s="43"/>
-      <c r="BB3" s="44"/>
-      <c r="BC3" s="42" t="e" vm="7">
+      <c r="BA3" s="41"/>
+      <c r="BB3" s="42"/>
+      <c r="BC3" s="40" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD3" s="43"/>
-      <c r="BE3" s="44"/>
-      <c r="BF3" s="42" t="e" vm="14">
+      <c r="BD3" s="41"/>
+      <c r="BE3" s="42"/>
+      <c r="BF3" s="40" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG3" s="43"/>
-      <c r="BH3" s="44"/>
-      <c r="BI3" s="39" t="e" vm="15">
+      <c r="BG3" s="41"/>
+      <c r="BH3" s="42"/>
+      <c r="BI3" s="37" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ3" s="40"/>
-      <c r="BK3" s="40"/>
-      <c r="BL3" s="40"/>
-      <c r="BM3" s="41"/>
-      <c r="BN3" s="42" t="e" vm="4">
+      <c r="BJ3" s="38"/>
+      <c r="BK3" s="38"/>
+      <c r="BL3" s="38"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="40" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO3" s="43"/>
-      <c r="BP3" s="44"/>
-      <c r="BQ3" s="42" t="e" vm="16">
+      <c r="BO3" s="41"/>
+      <c r="BP3" s="42"/>
+      <c r="BQ3" s="40" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR3" s="43"/>
-      <c r="BS3" s="44"/>
-      <c r="BT3" s="42" t="e" vm="17">
+      <c r="BR3" s="41"/>
+      <c r="BS3" s="42"/>
+      <c r="BT3" s="40" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU3" s="43"/>
-      <c r="BV3" s="44"/>
-      <c r="BW3" s="42" t="e" vm="4">
+      <c r="BU3" s="41"/>
+      <c r="BV3" s="42"/>
+      <c r="BW3" s="40" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX3" s="43"/>
-      <c r="BY3" s="44"/>
-      <c r="BZ3" s="42" t="e" vm="18">
+      <c r="BX3" s="41"/>
+      <c r="BY3" s="42"/>
+      <c r="BZ3" s="40" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA3" s="43"/>
-      <c r="CB3" s="44"/>
-      <c r="CC3" s="42" t="e" vm="19">
+      <c r="CA3" s="41"/>
+      <c r="CB3" s="42"/>
+      <c r="CC3" s="40" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD3" s="43"/>
-      <c r="CE3" s="44"/>
+      <c r="CD3" s="41"/>
+      <c r="CE3" s="42"/>
     </row>
     <row r="4" spans="1:83" s="16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="32" t="s">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="E10" s="2" cm="1">
         <f t="array" ref="E10">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H10,M10,P10,U10,Z10,AC10,AF10,AI10,AN10,AQ10,AT10,AY10,BB10,BE10,BH10,BM10,BP10,BS10,BV10,BY10,CB10,CE10), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.99</v>
+        <v>0.69599999999999995</v>
       </c>
       <c r="F10" s="21">
         <v>0</v>
@@ -4586,7 +4586,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="28">
-        <v>8.25</v>
+        <v>5.8</v>
       </c>
       <c r="W10" s="23">
         <v>0</v>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="Z10" s="24">
         <f t="shared" si="4"/>
-        <v>0.99</v>
+        <v>0.69599999999999995</v>
       </c>
       <c r="AA10" s="28">
         <v>0</v>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="E11" s="2" cm="1">
         <f t="array" ref="E11">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H11,M11,P11,U11,Z11,AC11,AF11,AI11,AN11,AQ11,AT11,AY11,BB11,BE11,BH11,BM11,BP11,BS11,BV11,BY11,CB11,CE11), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.69599999999999995</v>
+        <v>0.99</v>
       </c>
       <c r="F11" s="21">
         <v>0</v>
@@ -4860,7 +4860,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="28">
-        <v>5.8</v>
+        <v>8.25</v>
       </c>
       <c r="W11" s="23">
         <v>0</v>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="Z11" s="24">
         <f t="shared" si="4"/>
-        <v>0.69599999999999995</v>
+        <v>0.99</v>
       </c>
       <c r="AA11" s="28">
         <v>0</v>
@@ -9458,150 +9458,150 @@
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
-      <c r="F29" s="39" t="e" vm="1">
+      <c r="F29" s="37" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G29" s="40"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="40" t="e" vm="2">
+      <c r="G29" s="38"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="38" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="40"/>
-      <c r="M29" s="40"/>
-      <c r="N29" s="39" t="e" vm="3">
+      <c r="J29" s="38"/>
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="37" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O29" s="40"/>
-      <c r="P29" s="41"/>
-      <c r="Q29" s="40" t="e" vm="4">
+      <c r="O29" s="38"/>
+      <c r="P29" s="39"/>
+      <c r="Q29" s="38" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R29" s="40"/>
-      <c r="S29" s="40"/>
-      <c r="T29" s="40"/>
-      <c r="U29" s="41"/>
-      <c r="V29" s="39" t="e" vm="5">
+      <c r="R29" s="38"/>
+      <c r="S29" s="38"/>
+      <c r="T29" s="38"/>
+      <c r="U29" s="39"/>
+      <c r="V29" s="37" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W29" s="40"/>
-      <c r="X29" s="40"/>
-      <c r="Y29" s="40"/>
-      <c r="Z29" s="40"/>
-      <c r="AA29" s="39" t="e" vm="6">
+      <c r="W29" s="38"/>
+      <c r="X29" s="38"/>
+      <c r="Y29" s="38"/>
+      <c r="Z29" s="38"/>
+      <c r="AA29" s="37" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB29" s="40"/>
-      <c r="AC29" s="41"/>
-      <c r="AD29" s="39" t="e" vm="7">
+      <c r="AB29" s="38"/>
+      <c r="AC29" s="39"/>
+      <c r="AD29" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE29" s="40"/>
-      <c r="AF29" s="41"/>
-      <c r="AG29" s="39" t="e" vm="8">
+      <c r="AE29" s="38"/>
+      <c r="AF29" s="39"/>
+      <c r="AG29" s="37" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH29" s="40"/>
-      <c r="AI29" s="41"/>
-      <c r="AJ29" s="40" t="e" vm="9">
+      <c r="AH29" s="38"/>
+      <c r="AI29" s="39"/>
+      <c r="AJ29" s="38" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK29" s="40"/>
-      <c r="AL29" s="40"/>
-      <c r="AM29" s="40"/>
-      <c r="AN29" s="40"/>
-      <c r="AO29" s="39" t="e" vm="10">
+      <c r="AK29" s="38"/>
+      <c r="AL29" s="38"/>
+      <c r="AM29" s="38"/>
+      <c r="AN29" s="38"/>
+      <c r="AO29" s="37" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP29" s="40"/>
-      <c r="AQ29" s="41"/>
-      <c r="AR29" s="39" t="e" vm="11">
+      <c r="AP29" s="38"/>
+      <c r="AQ29" s="39"/>
+      <c r="AR29" s="37" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS29" s="40"/>
-      <c r="AT29" s="41"/>
-      <c r="AU29" s="40" t="e" vm="12">
+      <c r="AS29" s="38"/>
+      <c r="AT29" s="39"/>
+      <c r="AU29" s="38" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV29" s="40"/>
-      <c r="AW29" s="40"/>
-      <c r="AX29" s="40"/>
-      <c r="AY29" s="40"/>
-      <c r="AZ29" s="39" t="e" vm="13">
+      <c r="AV29" s="38"/>
+      <c r="AW29" s="38"/>
+      <c r="AX29" s="38"/>
+      <c r="AY29" s="38"/>
+      <c r="AZ29" s="37" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA29" s="40"/>
-      <c r="BB29" s="41"/>
-      <c r="BC29" s="39" t="e" vm="7">
+      <c r="BA29" s="38"/>
+      <c r="BB29" s="39"/>
+      <c r="BC29" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD29" s="40"/>
-      <c r="BE29" s="41"/>
-      <c r="BF29" s="39" t="e" vm="14">
+      <c r="BD29" s="38"/>
+      <c r="BE29" s="39"/>
+      <c r="BF29" s="37" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG29" s="40"/>
-      <c r="BH29" s="41"/>
-      <c r="BI29" s="40" t="e" vm="15">
+      <c r="BG29" s="38"/>
+      <c r="BH29" s="39"/>
+      <c r="BI29" s="38" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ29" s="40"/>
-      <c r="BK29" s="40"/>
-      <c r="BL29" s="40"/>
-      <c r="BM29" s="40"/>
-      <c r="BN29" s="39" t="e" vm="4">
+      <c r="BJ29" s="38"/>
+      <c r="BK29" s="38"/>
+      <c r="BL29" s="38"/>
+      <c r="BM29" s="38"/>
+      <c r="BN29" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO29" s="40"/>
-      <c r="BP29" s="41"/>
-      <c r="BQ29" s="39" t="e" vm="16">
+      <c r="BO29" s="38"/>
+      <c r="BP29" s="39"/>
+      <c r="BQ29" s="37" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR29" s="40"/>
-      <c r="BS29" s="41"/>
-      <c r="BT29" s="39" t="e" vm="17">
+      <c r="BR29" s="38"/>
+      <c r="BS29" s="39"/>
+      <c r="BT29" s="37" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU29" s="40"/>
-      <c r="BV29" s="41"/>
-      <c r="BW29" s="39" t="e" vm="4">
+      <c r="BU29" s="38"/>
+      <c r="BV29" s="39"/>
+      <c r="BW29" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX29" s="40"/>
-      <c r="BY29" s="41"/>
-      <c r="BZ29" s="39" t="e" vm="18">
+      <c r="BX29" s="38"/>
+      <c r="BY29" s="39"/>
+      <c r="BZ29" s="37" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA29" s="40"/>
-      <c r="CB29" s="41"/>
-      <c r="CC29" s="39" t="e" vm="19">
+      <c r="CA29" s="38"/>
+      <c r="CB29" s="39"/>
+      <c r="CC29" s="37" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD29" s="40"/>
-      <c r="CE29" s="41"/>
+      <c r="CD29" s="38"/>
+      <c r="CE29" s="39"/>
     </row>
     <row r="30" spans="1:83" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="32" t="s">
@@ -11495,10 +11495,10 @@
         <v>7</v>
       </c>
       <c r="B38" s="4">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C38" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Lewis Hamilton</v>
       </c>
       <c r="D38" s="4" t="str">
         <v>Ferrari</v>
@@ -14758,10 +14758,10 @@
         <v>20</v>
       </c>
       <c r="B51" s="10">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="C51" s="12" t="str">
-        <v>Lewis Hamilton</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D51" s="10" t="str">
         <v>Ferrari</v>
@@ -15532,28 +15532,67 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="I30:M30"/>
-    <mergeCell ref="N30:P30"/>
-    <mergeCell ref="BW30:BY30"/>
-    <mergeCell ref="BZ30:CB30"/>
-    <mergeCell ref="Q30:U30"/>
-    <mergeCell ref="V30:Z30"/>
-    <mergeCell ref="AA30:AC30"/>
-    <mergeCell ref="AD30:AF30"/>
-    <mergeCell ref="AG30:AI30"/>
-    <mergeCell ref="AJ30:AN30"/>
-    <mergeCell ref="AO30:AQ30"/>
-    <mergeCell ref="AR30:AT30"/>
-    <mergeCell ref="AU30:AY30"/>
-    <mergeCell ref="CC30:CE30"/>
-    <mergeCell ref="AZ30:BB30"/>
-    <mergeCell ref="BC30:BE30"/>
-    <mergeCell ref="BF30:BH30"/>
-    <mergeCell ref="BI30:BM30"/>
-    <mergeCell ref="BN30:BP30"/>
-    <mergeCell ref="BQ30:BS30"/>
-    <mergeCell ref="BT30:BV30"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="Q3:U3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="N29:P29"/>
+    <mergeCell ref="Q29:U29"/>
+    <mergeCell ref="V29:Z29"/>
+    <mergeCell ref="V4:Z4"/>
+    <mergeCell ref="AG3:AI3"/>
+    <mergeCell ref="AJ3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="AA4:AC4"/>
+    <mergeCell ref="AD4:AF4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="AJ4:AN4"/>
+    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="BW3:BY3"/>
+    <mergeCell ref="BZ3:CB3"/>
+    <mergeCell ref="CC3:CE3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="V3:Z3"/>
+    <mergeCell ref="AA3:AC3"/>
+    <mergeCell ref="AD3:AF3"/>
+    <mergeCell ref="BT3:BV3"/>
+    <mergeCell ref="AU3:AY3"/>
+    <mergeCell ref="AZ3:BB3"/>
+    <mergeCell ref="BC3:BE3"/>
+    <mergeCell ref="BF3:BH3"/>
+    <mergeCell ref="BI3:BM3"/>
+    <mergeCell ref="BN3:BP3"/>
+    <mergeCell ref="BQ3:BS3"/>
+    <mergeCell ref="CC4:CE4"/>
+    <mergeCell ref="AR4:AT4"/>
+    <mergeCell ref="AU4:AY4"/>
+    <mergeCell ref="AZ4:BB4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="BF4:BH4"/>
+    <mergeCell ref="BI4:BM4"/>
+    <mergeCell ref="BN4:BP4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BT4:BV4"/>
+    <mergeCell ref="BW4:BY4"/>
+    <mergeCell ref="BZ4:CB4"/>
+    <mergeCell ref="BQ29:BS29"/>
+    <mergeCell ref="BT29:BV29"/>
+    <mergeCell ref="AG29:AI29"/>
+    <mergeCell ref="AJ29:AN29"/>
+    <mergeCell ref="AO29:AQ29"/>
+    <mergeCell ref="AR29:AT29"/>
     <mergeCell ref="BW29:BY29"/>
     <mergeCell ref="BZ29:CB29"/>
     <mergeCell ref="CC29:CE29"/>
@@ -15570,67 +15609,28 @@
     <mergeCell ref="BN29:BP29"/>
     <mergeCell ref="AA29:AC29"/>
     <mergeCell ref="AD29:AF29"/>
-    <mergeCell ref="BQ29:BS29"/>
-    <mergeCell ref="BT29:BV29"/>
-    <mergeCell ref="AG29:AI29"/>
-    <mergeCell ref="AJ29:AN29"/>
-    <mergeCell ref="AO29:AQ29"/>
-    <mergeCell ref="CC4:CE4"/>
-    <mergeCell ref="AR4:AT4"/>
-    <mergeCell ref="AU4:AY4"/>
-    <mergeCell ref="AZ4:BB4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="BF4:BH4"/>
-    <mergeCell ref="BI4:BM4"/>
-    <mergeCell ref="BN4:BP4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BT4:BV4"/>
-    <mergeCell ref="BW4:BY4"/>
-    <mergeCell ref="BZ4:CB4"/>
-    <mergeCell ref="BW3:BY3"/>
-    <mergeCell ref="BZ3:CB3"/>
-    <mergeCell ref="CC3:CE3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="V3:Z3"/>
-    <mergeCell ref="AA3:AC3"/>
-    <mergeCell ref="AD3:AF3"/>
-    <mergeCell ref="BT3:BV3"/>
-    <mergeCell ref="AU3:AY3"/>
-    <mergeCell ref="AZ3:BB3"/>
-    <mergeCell ref="BC3:BE3"/>
-    <mergeCell ref="BF3:BH3"/>
-    <mergeCell ref="BI3:BM3"/>
-    <mergeCell ref="BN3:BP3"/>
-    <mergeCell ref="BQ3:BS3"/>
-    <mergeCell ref="V4:Z4"/>
-    <mergeCell ref="AG3:AI3"/>
-    <mergeCell ref="AJ3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="AR29:AT29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="N29:P29"/>
-    <mergeCell ref="Q29:U29"/>
-    <mergeCell ref="V29:Z29"/>
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="Q3:U3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="AA4:AC4"/>
-    <mergeCell ref="AD4:AF4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="AJ4:AN4"/>
-    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="CC30:CE30"/>
+    <mergeCell ref="AZ30:BB30"/>
+    <mergeCell ref="BC30:BE30"/>
+    <mergeCell ref="BF30:BH30"/>
+    <mergeCell ref="BI30:BM30"/>
+    <mergeCell ref="BN30:BP30"/>
+    <mergeCell ref="BQ30:BS30"/>
+    <mergeCell ref="BT30:BV30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:M30"/>
+    <mergeCell ref="N30:P30"/>
+    <mergeCell ref="BW30:BY30"/>
+    <mergeCell ref="BZ30:CB30"/>
+    <mergeCell ref="Q30:U30"/>
+    <mergeCell ref="V30:Z30"/>
+    <mergeCell ref="AA30:AC30"/>
+    <mergeCell ref="AD30:AF30"/>
+    <mergeCell ref="AG30:AI30"/>
+    <mergeCell ref="AJ30:AN30"/>
+    <mergeCell ref="AO30:AQ30"/>
+    <mergeCell ref="AR30:AT30"/>
+    <mergeCell ref="AU30:AY30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B27 D6:D27 B32:B53 D32:D53">
     <cfRule type="expression" dxfId="65" priority="329">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="N4" s="29">
         <f>Simplified!G6</f>
-        <v>0.29400000000000004</v>
+        <v>-0.29400000000000004</v>
       </c>
       <c r="O4" s="3">
         <v>44</v>
@@ -15986,7 +15986,7 @@
       </c>
       <c r="G6" s="45">
         <f>K6-K7</f>
-        <v>0.29400000000000004</v>
+        <v>-0.29400000000000004</v>
       </c>
       <c r="H6" s="3">
         <v>16</v>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="K6" s="2">
         <f>Ratings!E10</f>
-        <v>0.99</v>
+        <v>0.69599999999999995</v>
       </c>
       <c r="M6" s="5">
         <v>10</v>
@@ -16040,7 +16040,7 @@
       </c>
       <c r="K7" s="2">
         <f>Ratings!E11</f>
-        <v>0.69599999999999995</v>
+        <v>0.99</v>
       </c>
       <c r="M7" s="6">
         <v>30</v>
@@ -16058,10 +16058,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C8" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Lewis Hamilton</v>
       </c>
       <c r="D8" s="4" t="str">
         <v>Ferrari</v>
@@ -16532,10 +16532,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="10">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="C21" s="12" t="str">
-        <v>Lewis Hamilton</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D21" s="10" t="str">
         <v>Ferrari</v>
@@ -16684,7 +16684,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2 G4 G6 G8 G10 G12 G14 G16 G18 G20 G22">
+  <conditionalFormatting sqref="G4 G2 G6 G8 G10 G12 G14 G16 G18 G20 G22">
     <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="percentile" val="0"/>

</xml_diff>

<commit_message>
corrected sq info only
</commit_message>
<xml_diff>
--- a/static/data/Ratings.xlsx
+++ b/static/data/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Programming\webdev\portfolio\static\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB68969A-3BD9-4485-8BE5-55D3B8DFED46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DFC0EF-5CD6-4E8E-A821-A92654F377E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="2" activeTab="2" xr2:uid="{BD88BCC4-2E11-4C36-830D-A75A044EF5A6}"/>
   </bookViews>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="E8" s="2" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H8,M8,P8,U8,Z8,AC8,AF8,AI8,AN8,AQ8,AT8,AY8,BB8,BE8,BH8,BM8,BP8,BS8,BV8,BY8,CB8,CE8), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="F8" s="21">
         <v>0</v>
@@ -4041,17 +4041,17 @@
         <v>8.75</v>
       </c>
       <c r="W8" s="23">
-        <v>9.8000000000000007</v>
+        <v>0</v>
       </c>
       <c r="X8" s="23">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="23">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="24">
         <f t="shared" si="4"/>
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="AA8" s="28">
         <v>0</v>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="E9" s="2" cm="1">
         <f t="array" ref="E9">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H9,M9,P9,U9,Z9,AC9,AF9,AI9,AN9,AQ9,AT9,AY9,BB9,BE9,BH9,BM9,BP9,BS9,BV9,BY9,CB9,CE9), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>5.827</v>
+        <v>1.02</v>
       </c>
       <c r="F9" s="21">
         <v>0</v>
@@ -4315,17 +4315,17 @@
         <v>8.5</v>
       </c>
       <c r="W9" s="23">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="X9" s="23">
-        <v>8.25</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="24">
         <f t="shared" si="4"/>
-        <v>5.827</v>
+        <v>1.02</v>
       </c>
       <c r="AA9" s="28">
         <v>0</v>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="E10" s="2" cm="1">
         <f t="array" ref="E10">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H10,M10,P10,U10,Z10,AC10,AF10,AI10,AN10,AQ10,AT10,AY10,BB10,BE10,BH10,BM10,BP10,BS10,BV10,BY10,CB10,CE10), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.69599999999999995</v>
+        <v>0.72</v>
       </c>
       <c r="F10" s="21">
         <v>0</v>
@@ -4586,7 +4586,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="28">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="W10" s="23">
         <v>0</v>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="Z10" s="24">
         <f t="shared" si="4"/>
-        <v>0.69599999999999995</v>
+        <v>0.72</v>
       </c>
       <c r="AA10" s="28">
         <v>0</v>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="E14" s="2" cm="1">
         <f t="array" ref="E14">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H14,M14,P14,U14,Z14,AC14,AF14,AI14,AN14,AQ14,AT14,AY14,BB14,BE14,BH14,BM14,BP14,BS14,BV14,BY14,CB14,CE14), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="F14" s="21">
         <v>0</v>
@@ -5682,7 +5682,7 @@
         <v>0</v>
       </c>
       <c r="V14" s="28">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="W14" s="23">
         <v>0</v>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="Z14" s="24">
         <f t="shared" si="4"/>
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="AA14" s="28">
         <v>0</v>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="E15" s="2" cm="1">
         <f t="array" ref="E15">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H15,M15,P15,U15,Z15,AC15,AF15,AI15,AN15,AQ15,AT15,AY15,BB15,BE15,BH15,BM15,BP15,BS15,BV15,BY15,CB15,CE15), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="F15" s="21">
         <v>0</v>
@@ -5956,7 +5956,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="28">
-        <v>8.5</v>
+        <v>8.75</v>
       </c>
       <c r="W15" s="23">
         <v>0</v>
@@ -5969,7 +5969,7 @@
       </c>
       <c r="Z15" s="24">
         <f t="shared" si="4"/>
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="AA15" s="28">
         <v>0</v>
@@ -8366,7 +8366,7 @@
       </c>
       <c r="E24" s="2" cm="1">
         <f t="array" ref="E24">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H24,M24,P24,U24,Z24,AC24,AF24,AI24,AN24,AQ24,AT24,AY24,BB24,BE24,BH24,BM24,BP24,BS24,BV24,BY24,CB24,CE24), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
       <c r="F24" s="21">
         <v>0</v>
@@ -8420,7 +8420,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="28">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="W24" s="23">
         <v>0</v>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="Z24" s="24">
         <f t="shared" si="4"/>
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
       <c r="AA24" s="28">
         <v>0</v>
@@ -9187,7 +9187,7 @@
       </c>
       <c r="E27" s="2" cm="1">
         <f t="array" ref="E27">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H27,M27,P27,U27,Z27,AC27,AF27,AI27,AN27,AQ27,AT27,AY27,BB27,BE27,BH27,BM27,BP27,BS27,BV27,BY27,CB27,CE27), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
       <c r="F27" s="21">
         <v>0</v>
@@ -9242,7 +9242,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W27" s="23">
         <v>0</v>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="Z27" s="24">
         <f t="shared" si="4"/>
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
       <c r="AA27" s="28">
         <v>0</v>
@@ -9998,7 +9998,7 @@
         <v>McLaren</v>
       </c>
       <c r="E32" s="2">
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="F32" s="21">
         <v>0</v>
@@ -10052,16 +10052,16 @@
         <v>8.75</v>
       </c>
       <c r="W32" s="23">
-        <v>9.8000000000000007</v>
+        <v>0</v>
       </c>
       <c r="X32" s="23">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="Y32" s="23">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="Z32" s="24">
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="AA32" s="28">
         <v>0</v>
@@ -10240,16 +10240,16 @@
         <v>2</v>
       </c>
       <c r="B33" s="18">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="C33" s="12" t="str">
-        <v>Oscar Piastri</v>
+        <v>Franco Colapinto</v>
       </c>
       <c r="D33" s="18" t="str">
-        <v>McLaren</v>
+        <v>Alpine</v>
       </c>
       <c r="E33" s="2">
-        <v>5.827</v>
+        <v>1.05</v>
       </c>
       <c r="F33" s="21">
         <v>0</v>
@@ -10300,19 +10300,19 @@
         <v>0</v>
       </c>
       <c r="V33" s="28">
-        <v>8.5</v>
+        <v>8.75</v>
       </c>
       <c r="W33" s="23">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="X33" s="23">
-        <v>8.25</v>
+        <v>0</v>
       </c>
       <c r="Y33" s="23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z33" s="24">
-        <v>5.827</v>
+        <v>1.05</v>
       </c>
       <c r="AA33" s="28">
         <v>0</v>
@@ -10742,13 +10742,13 @@
         <v>4</v>
       </c>
       <c r="B35" s="1">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="C35" s="12" t="str">
-        <v>Franco Colapinto</v>
+        <v>Oscar Piastri</v>
       </c>
       <c r="D35" s="1" t="str">
-        <v>Alpine</v>
+        <v>McLaren</v>
       </c>
       <c r="E35" s="2">
         <v>1.02</v>
@@ -11244,16 +11244,16 @@
         <v>6</v>
       </c>
       <c r="B37" s="3">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="C37" s="12" t="str">
-        <v>Sergio Perez</v>
+        <v>Lewis Hamilton</v>
       </c>
       <c r="D37" s="3" t="str">
-        <v>Cadillac</v>
+        <v>Ferrari</v>
       </c>
       <c r="E37" s="2">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="F37" s="21">
         <v>0</v>
@@ -11304,7 +11304,7 @@
         <v>0</v>
       </c>
       <c r="V37" s="28">
-        <v>8.5</v>
+        <v>8.25</v>
       </c>
       <c r="W37" s="23">
         <v>0</v>
@@ -11316,7 +11316,7 @@
         <v>0</v>
       </c>
       <c r="Z37" s="24">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="AA37" s="28">
         <v>0</v>
@@ -11495,16 +11495,16 @@
         <v>7</v>
       </c>
       <c r="B38" s="4">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C38" s="12" t="str">
-        <v>Lewis Hamilton</v>
+        <v>Kimi Antonelli</v>
       </c>
       <c r="D38" s="4" t="str">
-        <v>Ferrari</v>
+        <v>Mercedes</v>
       </c>
       <c r="E38" s="2">
-        <v>0.99</v>
+        <v>0.96</v>
       </c>
       <c r="F38" s="21">
         <v>0</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="V38" s="28">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="W38" s="23">
         <v>0</v>
@@ -11567,7 +11567,7 @@
         <v>0</v>
       </c>
       <c r="Z38" s="24">
-        <v>0.99</v>
+        <v>0.96</v>
       </c>
       <c r="AA38" s="28">
         <v>0</v>
@@ -11746,13 +11746,13 @@
         <v>8</v>
       </c>
       <c r="B39" s="4">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C39" s="12" t="str">
-        <v>Kimi Antonelli</v>
+        <v>Nico Hulkenberg</v>
       </c>
       <c r="D39" s="4" t="str">
-        <v>Mercedes</v>
+        <v>Audi</v>
       </c>
       <c r="E39" s="2">
         <v>0.96</v>
@@ -11997,13 +11997,13 @@
         <v>9</v>
       </c>
       <c r="B40" s="5">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="C40" s="12" t="str">
-        <v>Nico Hulkenberg</v>
+        <v>Sergio Perez</v>
       </c>
       <c r="D40" s="5" t="str">
-        <v>Audi</v>
+        <v>Cadillac</v>
       </c>
       <c r="E40" s="2">
         <v>0.96</v>
@@ -14507,13 +14507,13 @@
         <v>19</v>
       </c>
       <c r="B50" s="10">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C50" s="12" t="str">
-        <v>Lance Stroll</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D50" s="10" t="str">
-        <v>Aston Martin</v>
+        <v>Ferrari</v>
       </c>
       <c r="E50" s="2">
         <v>0.72</v>
@@ -14758,16 +14758,16 @@
         <v>20</v>
       </c>
       <c r="B51" s="10">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C51" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Lance Stroll</v>
       </c>
       <c r="D51" s="10" t="str">
-        <v>Ferrari</v>
+        <v>Aston Martin</v>
       </c>
       <c r="E51" s="2">
-        <v>0.69599999999999995</v>
+        <v>0.6</v>
       </c>
       <c r="F51" s="21">
         <v>0</v>
@@ -14818,7 +14818,7 @@
         <v>0</v>
       </c>
       <c r="V51" s="28">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="W51" s="23">
         <v>0</v>
@@ -14830,7 +14830,7 @@
         <v>0</v>
       </c>
       <c r="Z51" s="24">
-        <v>0.69599999999999995</v>
+        <v>0.6</v>
       </c>
       <c r="AA51" s="28">
         <v>0</v>
@@ -15018,7 +15018,7 @@
         <v>Alpine</v>
       </c>
       <c r="E52" s="2">
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="F52" s="21">
         <v>0</v>
@@ -15069,7 +15069,7 @@
         <v>0</v>
       </c>
       <c r="V52" s="28">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="W52" s="23">
         <v>0</v>
@@ -15081,7 +15081,7 @@
         <v>0</v>
       </c>
       <c r="Z52" s="24">
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="AA52" s="28">
         <v>0</v>
@@ -15812,7 +15812,7 @@
         <v>McLaren</v>
       </c>
       <c r="E2" s="2">
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="G2" s="45">
         <f>K2-K3</f>
@@ -15847,16 +15847,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="18">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="C3" s="12" t="str">
-        <v>Oscar Piastri</v>
+        <v>Franco Colapinto</v>
       </c>
       <c r="D3" s="18" t="str">
-        <v>McLaren</v>
+        <v>Alpine</v>
       </c>
       <c r="E3" s="2">
-        <v>5.827</v>
+        <v>1.05</v>
       </c>
       <c r="G3" s="45"/>
       <c r="H3" s="18">
@@ -15877,7 +15877,7 @@
       </c>
       <c r="N3" s="29">
         <f>Simplified!G4</f>
-        <v>2.859</v>
+        <v>3.0000000000000027E-2</v>
       </c>
       <c r="O3" s="1">
         <v>81</v>
@@ -15901,7 +15901,7 @@
       </c>
       <c r="G4" s="45">
         <f>K4-K5</f>
-        <v>2.859</v>
+        <v>3.0000000000000027E-2</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
@@ -15914,14 +15914,14 @@
       </c>
       <c r="K4" s="2">
         <f>Ratings!E8</f>
-        <v>8.6859999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="M4" s="3">
         <v>16</v>
       </c>
       <c r="N4" s="29">
         <f>Simplified!G6</f>
-        <v>-0.29400000000000004</v>
+        <v>-0.27</v>
       </c>
       <c r="O4" s="3">
         <v>44</v>
@@ -15932,13 +15932,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="C5" s="12" t="str">
-        <v>Franco Colapinto</v>
+        <v>Oscar Piastri</v>
       </c>
       <c r="D5" s="1" t="str">
-        <v>Alpine</v>
+        <v>McLaren</v>
       </c>
       <c r="E5" s="2">
         <v>1.02</v>
@@ -15955,7 +15955,7 @@
       </c>
       <c r="K5" s="2">
         <f>Ratings!E9</f>
-        <v>5.827</v>
+        <v>1.02</v>
       </c>
       <c r="M5" s="4">
         <v>3</v>
@@ -15986,7 +15986,7 @@
       </c>
       <c r="G6" s="45">
         <f>K6-K7</f>
-        <v>-0.29400000000000004</v>
+        <v>-0.27</v>
       </c>
       <c r="H6" s="3">
         <v>16</v>
@@ -15999,14 +15999,14 @@
       </c>
       <c r="K6" s="2">
         <f>Ratings!E10</f>
-        <v>0.69599999999999995</v>
+        <v>0.72</v>
       </c>
       <c r="M6" s="5">
         <v>10</v>
       </c>
       <c r="N6" s="29">
         <f>Simplified!G10</f>
-        <v>-0.54</v>
+        <v>-0.63000000000000012</v>
       </c>
       <c r="O6" s="5">
         <v>43</v>
@@ -16017,16 +16017,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="3">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="C7" s="12" t="str">
-        <v>Sergio Perez</v>
+        <v>Lewis Hamilton</v>
       </c>
       <c r="D7" s="3" t="str">
-        <v>Cadillac</v>
+        <v>Ferrari</v>
       </c>
       <c r="E7" s="2">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="G7" s="45"/>
       <c r="H7" s="3">
@@ -16058,16 +16058,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="4">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C8" s="12" t="str">
-        <v>Lewis Hamilton</v>
+        <v>Kimi Antonelli</v>
       </c>
       <c r="D8" s="4" t="str">
-        <v>Ferrari</v>
+        <v>Mercedes</v>
       </c>
       <c r="E8" s="2">
-        <v>0.99</v>
+        <v>0.96</v>
       </c>
       <c r="G8" s="45">
         <f>K8-K9</f>
@@ -16102,13 +16102,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C9" s="12" t="str">
-        <v>Kimi Antonelli</v>
+        <v>Nico Hulkenberg</v>
       </c>
       <c r="D9" s="4" t="str">
-        <v>Mercedes</v>
+        <v>Audi</v>
       </c>
       <c r="E9" s="2">
         <v>0.96</v>
@@ -16143,20 +16143,20 @@
         <v>9</v>
       </c>
       <c r="B10" s="5">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="C10" s="12" t="str">
-        <v>Nico Hulkenberg</v>
+        <v>Sergio Perez</v>
       </c>
       <c r="D10" s="5" t="str">
-        <v>Audi</v>
+        <v>Cadillac</v>
       </c>
       <c r="E10" s="2">
         <v>0.96</v>
       </c>
       <c r="G10" s="45">
         <f>K10-K11</f>
-        <v>-0.54</v>
+        <v>-0.63000000000000012</v>
       </c>
       <c r="H10" s="5">
         <v>10</v>
@@ -16169,7 +16169,7 @@
       </c>
       <c r="K10" s="2">
         <f>Ratings!E14</f>
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="M10" s="9">
         <v>27</v>
@@ -16210,14 +16210,14 @@
       </c>
       <c r="K11" s="2">
         <f>Ratings!E15</f>
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="M11" s="10">
         <v>11</v>
       </c>
       <c r="N11" s="29">
         <f>Simplified!G20</f>
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="O11" s="10">
         <v>77</v>
@@ -16261,7 +16261,7 @@
       </c>
       <c r="N12" s="29">
         <f>Simplified!G22</f>
-        <v>0.17999999999999994</v>
+        <v>0.29999999999999993</v>
       </c>
       <c r="O12" s="11">
         <v>18</v>
@@ -16498,20 +16498,20 @@
         <v>19</v>
       </c>
       <c r="B20" s="10">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C20" s="12" t="str">
-        <v>Lance Stroll</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D20" s="10" t="str">
-        <v>Aston Martin</v>
+        <v>Ferrari</v>
       </c>
       <c r="E20" s="2">
         <v>0.72</v>
       </c>
       <c r="G20" s="45">
         <f>K20-K21</f>
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="H20" s="10">
         <v>11</v>
@@ -16524,7 +16524,7 @@
       </c>
       <c r="K20" s="2">
         <f>Ratings!E24</f>
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
@@ -16532,16 +16532,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="10">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C21" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Lance Stroll</v>
       </c>
       <c r="D21" s="10" t="str">
-        <v>Ferrari</v>
+        <v>Aston Martin</v>
       </c>
       <c r="E21" s="2">
-        <v>0.69599999999999995</v>
+        <v>0.6</v>
       </c>
       <c r="G21" s="45"/>
       <c r="H21" s="10">
@@ -16572,11 +16572,11 @@
         <v>Alpine</v>
       </c>
       <c r="E22" s="2">
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="G22" s="45">
         <f>K22-K23</f>
-        <v>0.17999999999999994</v>
+        <v>0.29999999999999993</v>
       </c>
       <c r="H22" s="11">
         <v>14</v>
@@ -16620,7 +16620,7 @@
       </c>
       <c r="K23" s="2">
         <f>Ratings!E27</f>
-        <v>0.72</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
slept on it rankings changed
</commit_message>
<xml_diff>
--- a/static/data/Ratings.xlsx
+++ b/static/data/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Programming\webdev\portfolio\static\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DFC0EF-5CD6-4E8E-A821-A92654F377E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FE96B4-3B4B-4F42-AD69-28AF6C6412A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="2" activeTab="2" xr2:uid="{BD88BCC4-2E11-4C36-830D-A75A044EF5A6}"/>
   </bookViews>
@@ -259,7 +259,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="73">
   <si>
     <t>RANK</t>
   </si>
@@ -475,6 +475,9 @@
   </si>
   <si>
     <t>Dummy</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -906,10 +909,34 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -922,30 +949,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2718,13 +2721,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:83" s="14" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
       <c r="F1" s="17"/>
       <c r="G1" s="17"/>
       <c r="H1" s="17"/>
@@ -2805,11 +2808,11 @@
       <c r="CE1" s="17"/>
     </row>
     <row r="2" spans="1:83" s="14" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="44"/>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
       <c r="F2" s="17"/>
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
@@ -2895,296 +2898,296 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
-      <c r="F3" s="40" t="e" vm="1">
+      <c r="F3" s="37" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="38" t="e" vm="2">
+      <c r="G3" s="38"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="34" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="40" t="e" vm="3">
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="37" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O3" s="41"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="37" t="e" vm="4">
+      <c r="O3" s="38"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="33" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R3" s="38"/>
-      <c r="S3" s="38"/>
-      <c r="T3" s="38"/>
-      <c r="U3" s="39"/>
-      <c r="V3" s="37" t="e" vm="5">
+      <c r="R3" s="34"/>
+      <c r="S3" s="34"/>
+      <c r="T3" s="34"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="33" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W3" s="38"/>
-      <c r="X3" s="38"/>
-      <c r="Y3" s="38"/>
-      <c r="Z3" s="39"/>
-      <c r="AA3" s="40" t="e" vm="6">
+      <c r="W3" s="34"/>
+      <c r="X3" s="34"/>
+      <c r="Y3" s="34"/>
+      <c r="Z3" s="35"/>
+      <c r="AA3" s="37" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="42"/>
-      <c r="AD3" s="40" t="e" vm="7">
+      <c r="AB3" s="38"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE3" s="41"/>
-      <c r="AF3" s="42"/>
-      <c r="AG3" s="40" t="e" vm="8">
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="37" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH3" s="41"/>
-      <c r="AI3" s="42"/>
-      <c r="AJ3" s="37" t="e" vm="9">
+      <c r="AH3" s="38"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="33" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK3" s="38"/>
-      <c r="AL3" s="38"/>
-      <c r="AM3" s="38"/>
-      <c r="AN3" s="39"/>
-      <c r="AO3" s="40" t="e" vm="10">
+      <c r="AK3" s="34"/>
+      <c r="AL3" s="34"/>
+      <c r="AM3" s="34"/>
+      <c r="AN3" s="35"/>
+      <c r="AO3" s="37" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP3" s="41"/>
-      <c r="AQ3" s="42"/>
-      <c r="AR3" s="40" t="e" vm="11">
+      <c r="AP3" s="38"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="37" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS3" s="41"/>
-      <c r="AT3" s="42"/>
-      <c r="AU3" s="37" t="e" vm="12">
+      <c r="AS3" s="38"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="33" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV3" s="38"/>
-      <c r="AW3" s="38"/>
-      <c r="AX3" s="38"/>
-      <c r="AY3" s="39"/>
-      <c r="AZ3" s="40" t="e" vm="13">
+      <c r="AV3" s="34"/>
+      <c r="AW3" s="34"/>
+      <c r="AX3" s="34"/>
+      <c r="AY3" s="35"/>
+      <c r="AZ3" s="37" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA3" s="41"/>
-      <c r="BB3" s="42"/>
-      <c r="BC3" s="40" t="e" vm="7">
+      <c r="BA3" s="38"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="37" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD3" s="41"/>
-      <c r="BE3" s="42"/>
-      <c r="BF3" s="40" t="e" vm="14">
+      <c r="BD3" s="38"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="37" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG3" s="41"/>
-      <c r="BH3" s="42"/>
-      <c r="BI3" s="37" t="e" vm="15">
+      <c r="BG3" s="38"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="33" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ3" s="38"/>
-      <c r="BK3" s="38"/>
-      <c r="BL3" s="38"/>
-      <c r="BM3" s="39"/>
-      <c r="BN3" s="40" t="e" vm="4">
+      <c r="BJ3" s="34"/>
+      <c r="BK3" s="34"/>
+      <c r="BL3" s="34"/>
+      <c r="BM3" s="35"/>
+      <c r="BN3" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO3" s="41"/>
-      <c r="BP3" s="42"/>
-      <c r="BQ3" s="40" t="e" vm="16">
+      <c r="BO3" s="38"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="37" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR3" s="41"/>
-      <c r="BS3" s="42"/>
-      <c r="BT3" s="40" t="e" vm="17">
+      <c r="BR3" s="38"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="37" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU3" s="41"/>
-      <c r="BV3" s="42"/>
-      <c r="BW3" s="40" t="e" vm="4">
+      <c r="BU3" s="38"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="37" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX3" s="41"/>
-      <c r="BY3" s="42"/>
-      <c r="BZ3" s="40" t="e" vm="18">
+      <c r="BX3" s="38"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="37" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA3" s="41"/>
-      <c r="CB3" s="42"/>
-      <c r="CC3" s="40" t="e" vm="19">
+      <c r="CA3" s="38"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="37" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD3" s="41"/>
-      <c r="CE3" s="42"/>
+      <c r="CD3" s="38"/>
+      <c r="CE3" s="39"/>
     </row>
     <row r="4" spans="1:83" s="16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="32" t="s">
+      <c r="A4" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="32" t="s">
+      <c r="E4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="32"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="32" t="s">
+      <c r="G4" s="36"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="31" t="s">
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="O4" s="32"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="34" t="s">
+      <c r="O4" s="36"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="R4" s="35"/>
-      <c r="S4" s="35"/>
-      <c r="T4" s="35"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="34" t="s">
+      <c r="R4" s="43"/>
+      <c r="S4" s="43"/>
+      <c r="T4" s="43"/>
+      <c r="U4" s="44"/>
+      <c r="V4" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="W4" s="35"/>
-      <c r="X4" s="35"/>
-      <c r="Y4" s="35"/>
-      <c r="Z4" s="36"/>
-      <c r="AA4" s="31" t="s">
+      <c r="W4" s="43"/>
+      <c r="X4" s="43"/>
+      <c r="Y4" s="43"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="AB4" s="32"/>
-      <c r="AC4" s="33"/>
-      <c r="AD4" s="31" t="s">
+      <c r="AB4" s="36"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="AE4" s="32"/>
-      <c r="AF4" s="33"/>
-      <c r="AG4" s="31" t="s">
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="AH4" s="32"/>
-      <c r="AI4" s="33"/>
-      <c r="AJ4" s="34" t="s">
+      <c r="AH4" s="36"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="AK4" s="35"/>
-      <c r="AL4" s="35"/>
-      <c r="AM4" s="35"/>
-      <c r="AN4" s="36"/>
-      <c r="AO4" s="31" t="s">
+      <c r="AK4" s="43"/>
+      <c r="AL4" s="43"/>
+      <c r="AM4" s="43"/>
+      <c r="AN4" s="44"/>
+      <c r="AO4" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="AP4" s="32"/>
-      <c r="AQ4" s="33"/>
-      <c r="AR4" s="31" t="s">
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="AS4" s="32"/>
-      <c r="AT4" s="33"/>
-      <c r="AU4" s="34" t="s">
+      <c r="AS4" s="36"/>
+      <c r="AT4" s="41"/>
+      <c r="AU4" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="AV4" s="35"/>
-      <c r="AW4" s="35"/>
-      <c r="AX4" s="35"/>
-      <c r="AY4" s="36"/>
-      <c r="AZ4" s="31" t="s">
+      <c r="AV4" s="43"/>
+      <c r="AW4" s="43"/>
+      <c r="AX4" s="43"/>
+      <c r="AY4" s="44"/>
+      <c r="AZ4" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="BA4" s="32"/>
-      <c r="BB4" s="33"/>
-      <c r="BC4" s="31" t="s">
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="41"/>
+      <c r="BC4" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="BD4" s="32"/>
-      <c r="BE4" s="33"/>
-      <c r="BF4" s="31" t="s">
+      <c r="BD4" s="36"/>
+      <c r="BE4" s="41"/>
+      <c r="BF4" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="BG4" s="32"/>
-      <c r="BH4" s="33"/>
-      <c r="BI4" s="34" t="s">
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="41"/>
+      <c r="BI4" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="BJ4" s="35"/>
-      <c r="BK4" s="35"/>
-      <c r="BL4" s="35"/>
-      <c r="BM4" s="36"/>
-      <c r="BN4" s="31" t="s">
+      <c r="BJ4" s="43"/>
+      <c r="BK4" s="43"/>
+      <c r="BL4" s="43"/>
+      <c r="BM4" s="44"/>
+      <c r="BN4" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="BO4" s="32"/>
-      <c r="BP4" s="33"/>
-      <c r="BQ4" s="31" t="s">
+      <c r="BO4" s="36"/>
+      <c r="BP4" s="41"/>
+      <c r="BQ4" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="BR4" s="32"/>
-      <c r="BS4" s="33"/>
-      <c r="BT4" s="31" t="s">
+      <c r="BR4" s="36"/>
+      <c r="BS4" s="41"/>
+      <c r="BT4" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="BU4" s="32"/>
-      <c r="BV4" s="33"/>
-      <c r="BW4" s="31" t="s">
+      <c r="BU4" s="36"/>
+      <c r="BV4" s="41"/>
+      <c r="BW4" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="BX4" s="32"/>
-      <c r="BY4" s="33"/>
-      <c r="BZ4" s="31" t="s">
+      <c r="BX4" s="36"/>
+      <c r="BY4" s="41"/>
+      <c r="BZ4" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="CA4" s="32"/>
-      <c r="CB4" s="33"/>
-      <c r="CC4" s="31" t="s">
+      <c r="CA4" s="36"/>
+      <c r="CB4" s="41"/>
+      <c r="CC4" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="CD4" s="32"/>
-      <c r="CE4" s="33"/>
+      <c r="CD4" s="36"/>
+      <c r="CE4" s="41"/>
     </row>
     <row r="5" spans="1:83" s="16" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="32"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
       <c r="F5" s="22" t="s">
         <v>26</v>
       </c>
@@ -5353,7 +5356,7 @@
       </c>
       <c r="E13" s="2" cm="1">
         <f t="array" ref="E13">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H13,M13,P13,U13,Z13,AC13,AF13,AI13,AN13,AQ13,AT13,AY13,BB13,BE13,BH13,BM13,BP13,BS13,BV13,BY13,CB13,CE13), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.89999999999999991</v>
+        <v>0.87</v>
       </c>
       <c r="F13" s="21">
         <v>0</v>
@@ -5408,7 +5411,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="28">
-        <v>7.5</v>
+        <v>7.25</v>
       </c>
       <c r="W13" s="23">
         <v>0</v>
@@ -5421,7 +5424,7 @@
       </c>
       <c r="Z13" s="24">
         <f t="shared" si="4"/>
-        <v>0.89999999999999991</v>
+        <v>0.87</v>
       </c>
       <c r="AA13" s="28">
         <v>0</v>
@@ -6175,7 +6178,7 @@
       </c>
       <c r="E16" s="2" cm="1">
         <f t="array" ref="E16">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H16,M16,P16,U16,Z16,AC16,AF16,AI16,AN16,AQ16,AT16,AY16,BB16,BE16,BH16,BM16,BP16,BS16,BV16,BY16,CB16,CE16), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="F16" s="21">
         <v>0</v>
@@ -6229,8 +6232,8 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="V16" s="28">
-        <v>7</v>
+      <c r="V16" s="28" t="s">
+        <v>72</v>
       </c>
       <c r="W16" s="23">
         <v>0</v>
@@ -6243,7 +6246,7 @@
       </c>
       <c r="Z16" s="24">
         <f t="shared" si="4"/>
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="28">
         <v>0</v>
@@ -6449,7 +6452,7 @@
       </c>
       <c r="E17" s="2" cm="1">
         <f t="array" ref="E17">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H17,M17,P17,U17,Z17,AC17,AF17,AI17,AN17,AQ17,AT17,AY17,BB17,BE17,BH17,BM17,BP17,BS17,BV17,BY17,CB17,CE17), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="F17" s="21">
         <v>0</v>
@@ -6504,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="V17" s="28">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
       <c r="W17" s="23">
         <v>0</v>
@@ -6517,7 +6520,7 @@
       </c>
       <c r="Z17" s="24">
         <f t="shared" si="4"/>
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="AA17" s="28">
         <v>0</v>
@@ -6997,7 +7000,7 @@
       </c>
       <c r="E19" s="2" cm="1">
         <f t="array" ref="E19">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H19,M19,P19,U19,Z19,AC19,AF19,AI19,AN19,AQ19,AT19,AY19,BB19,BE19,BH19,BM19,BP19,BS19,BV19,BY19,CB19,CE19), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="F19" s="21">
         <v>0</v>
@@ -7052,7 +7055,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="28">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="W19" s="23">
         <v>0</v>
@@ -7065,7 +7068,7 @@
       </c>
       <c r="Z19" s="24">
         <f t="shared" si="4"/>
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="AA19" s="28">
         <v>0</v>
@@ -7545,7 +7548,7 @@
       </c>
       <c r="E21" s="2" cm="1">
         <f t="array" ref="E21">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H21,M21,P21,U21,Z21,AC21,AF21,AI21,AN21,AQ21,AT21,AY21,BB21,BE21,BH21,BM21,BP21,BS21,BV21,BY21,CB21,CE21), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="F21" s="21">
         <v>0</v>
@@ -7599,8 +7602,8 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="V21" s="28">
-        <v>7</v>
+      <c r="V21" s="28" t="s">
+        <v>72</v>
       </c>
       <c r="W21" s="23">
         <v>0</v>
@@ -7613,7 +7616,7 @@
       </c>
       <c r="Z21" s="24">
         <f t="shared" si="4"/>
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="28">
         <v>0</v>
@@ -8092,7 +8095,7 @@
       </c>
       <c r="E23" s="2" cm="1">
         <f t="array" ref="E23">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H23,M23,P23,U23,Z23,AC23,AF23,AI23,AN23,AQ23,AT23,AY23,BB23,BE23,BH23,BM23,BP23,BS23,BV23,BY23,CB23,CE23), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.89400000000000002</v>
+        <v>0.89999999999999991</v>
       </c>
       <c r="F23" s="21">
         <v>0</v>
@@ -8147,7 +8150,7 @@
         <v>0</v>
       </c>
       <c r="V23" s="28">
-        <v>7.45</v>
+        <v>7.5</v>
       </c>
       <c r="W23" s="23">
         <v>0</v>
@@ -8160,7 +8163,7 @@
       </c>
       <c r="Z23" s="24">
         <f t="shared" si="4"/>
-        <v>0.89400000000000002</v>
+        <v>0.89999999999999991</v>
       </c>
       <c r="AA23" s="28">
         <v>0</v>
@@ -8366,7 +8369,7 @@
       </c>
       <c r="E24" s="2" cm="1">
         <f t="array" ref="E24">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H24,M24,P24,U24,Z24,AC24,AF24,AI24,AN24,AQ24,AT24,AY24,BB24,BE24,BH24,BM24,BP24,BS24,BV24,BY24,CB24,CE24), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="F24" s="21">
         <v>0</v>
@@ -8420,7 +8423,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="28">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="W24" s="23">
         <v>0</v>
@@ -8433,7 +8436,7 @@
       </c>
       <c r="Z24" s="24">
         <f t="shared" si="4"/>
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="AA24" s="28">
         <v>0</v>
@@ -8639,7 +8642,7 @@
       </c>
       <c r="E25" s="2" cm="1">
         <f t="array" ref="E25">_xlfn.LET(_xlpm.scores, _xlfn.VSTACK(H25,M25,P25,U25,Z25,AC25,AF25,AI25,AN25,AQ25,AT25,AY25,BB25,BE25,BH25,BM25,BP25,BS25,BV25,BY25,CB25,CE25), IFERROR(AVERAGE(_xlfn._xlws.FILTER(_xlpm.scores, _xlpm.scores&gt;0)), 0))</f>
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="F25" s="21">
         <v>0</v>
@@ -8694,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="28">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="W25" s="23">
         <v>0</v>
@@ -8707,7 +8710,7 @@
       </c>
       <c r="Z25" s="24">
         <f t="shared" si="4"/>
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="AA25" s="28">
         <v>0</v>
@@ -9458,296 +9461,296 @@
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
-      <c r="F29" s="37" t="e" vm="1">
+      <c r="F29" s="33" t="e" vm="1">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/au.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G29" s="38"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="38" t="e" vm="2">
+      <c r="G29" s="34"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="34" t="e" vm="2">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/cn.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J29" s="38"/>
-      <c r="K29" s="38"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="38"/>
-      <c r="N29" s="37" t="e" vm="3">
+      <c r="J29" s="34"/>
+      <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="33" t="e" vm="3">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/jp.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O29" s="38"/>
-      <c r="P29" s="39"/>
-      <c r="Q29" s="38" t="e" vm="4">
+      <c r="O29" s="34"/>
+      <c r="P29" s="35"/>
+      <c r="Q29" s="34" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R29" s="38"/>
-      <c r="S29" s="38"/>
-      <c r="T29" s="38"/>
-      <c r="U29" s="39"/>
-      <c r="V29" s="37" t="e" vm="5">
+      <c r="R29" s="34"/>
+      <c r="S29" s="34"/>
+      <c r="T29" s="34"/>
+      <c r="U29" s="35"/>
+      <c r="V29" s="33" t="e" vm="5">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ca.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W29" s="38"/>
-      <c r="X29" s="38"/>
-      <c r="Y29" s="38"/>
-      <c r="Z29" s="38"/>
-      <c r="AA29" s="37" t="e" vm="6">
+      <c r="W29" s="34"/>
+      <c r="X29" s="34"/>
+      <c r="Y29" s="34"/>
+      <c r="Z29" s="34"/>
+      <c r="AA29" s="33" t="e" vm="6">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mc.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AB29" s="38"/>
-      <c r="AC29" s="39"/>
-      <c r="AD29" s="37" t="e" vm="7">
+      <c r="AB29" s="34"/>
+      <c r="AC29" s="35"/>
+      <c r="AD29" s="33" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE29" s="38"/>
-      <c r="AF29" s="39"/>
-      <c r="AG29" s="37" t="e" vm="8">
+      <c r="AE29" s="34"/>
+      <c r="AF29" s="35"/>
+      <c r="AG29" s="33" t="e" vm="8">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/at.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AH29" s="38"/>
-      <c r="AI29" s="39"/>
-      <c r="AJ29" s="38" t="e" vm="9">
+      <c r="AH29" s="34"/>
+      <c r="AI29" s="35"/>
+      <c r="AJ29" s="34" t="e" vm="9">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/gb.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AK29" s="38"/>
-      <c r="AL29" s="38"/>
-      <c r="AM29" s="38"/>
-      <c r="AN29" s="38"/>
-      <c r="AO29" s="37" t="e" vm="10">
+      <c r="AK29" s="34"/>
+      <c r="AL29" s="34"/>
+      <c r="AM29" s="34"/>
+      <c r="AN29" s="34"/>
+      <c r="AO29" s="33" t="e" vm="10">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/be.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AP29" s="38"/>
-      <c r="AQ29" s="39"/>
-      <c r="AR29" s="37" t="e" vm="11">
+      <c r="AP29" s="34"/>
+      <c r="AQ29" s="35"/>
+      <c r="AR29" s="33" t="e" vm="11">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/hu.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AS29" s="38"/>
-      <c r="AT29" s="39"/>
-      <c r="AU29" s="38" t="e" vm="12">
+      <c r="AS29" s="34"/>
+      <c r="AT29" s="35"/>
+      <c r="AU29" s="34" t="e" vm="12">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/nl.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AV29" s="38"/>
-      <c r="AW29" s="38"/>
-      <c r="AX29" s="38"/>
-      <c r="AY29" s="38"/>
-      <c r="AZ29" s="37" t="e" vm="13">
+      <c r="AV29" s="34"/>
+      <c r="AW29" s="34"/>
+      <c r="AX29" s="34"/>
+      <c r="AY29" s="34"/>
+      <c r="AZ29" s="33" t="e" vm="13">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/it.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA29" s="38"/>
-      <c r="BB29" s="39"/>
-      <c r="BC29" s="37" t="e" vm="7">
+      <c r="BA29" s="34"/>
+      <c r="BB29" s="35"/>
+      <c r="BC29" s="33" t="e" vm="7">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/es.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BD29" s="38"/>
-      <c r="BE29" s="39"/>
-      <c r="BF29" s="37" t="e" vm="14">
+      <c r="BD29" s="34"/>
+      <c r="BE29" s="35"/>
+      <c r="BF29" s="33" t="e" vm="14">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/az.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BG29" s="38"/>
-      <c r="BH29" s="39"/>
-      <c r="BI29" s="38" t="e" vm="15">
+      <c r="BG29" s="34"/>
+      <c r="BH29" s="35"/>
+      <c r="BI29" s="34" t="e" vm="15">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/sg.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BJ29" s="38"/>
-      <c r="BK29" s="38"/>
-      <c r="BL29" s="38"/>
-      <c r="BM29" s="38"/>
-      <c r="BN29" s="37" t="e" vm="4">
+      <c r="BJ29" s="34"/>
+      <c r="BK29" s="34"/>
+      <c r="BL29" s="34"/>
+      <c r="BM29" s="34"/>
+      <c r="BN29" s="33" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BO29" s="38"/>
-      <c r="BP29" s="39"/>
-      <c r="BQ29" s="37" t="e" vm="16">
+      <c r="BO29" s="34"/>
+      <c r="BP29" s="35"/>
+      <c r="BQ29" s="33" t="e" vm="16">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/mx.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BR29" s="38"/>
-      <c r="BS29" s="39"/>
-      <c r="BT29" s="37" t="e" vm="17">
+      <c r="BR29" s="34"/>
+      <c r="BS29" s="35"/>
+      <c r="BT29" s="33" t="e" vm="17">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/br.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BU29" s="38"/>
-      <c r="BV29" s="39"/>
-      <c r="BW29" s="37" t="e" vm="4">
+      <c r="BU29" s="34"/>
+      <c r="BV29" s="35"/>
+      <c r="BW29" s="33" t="e" vm="4">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/us.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BX29" s="38"/>
-      <c r="BY29" s="39"/>
-      <c r="BZ29" s="37" t="e" vm="18">
+      <c r="BX29" s="34"/>
+      <c r="BY29" s="35"/>
+      <c r="BZ29" s="33" t="e" vm="18">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/qa.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CA29" s="38"/>
-      <c r="CB29" s="39"/>
-      <c r="CC29" s="37" t="e" vm="19">
+      <c r="CA29" s="34"/>
+      <c r="CB29" s="35"/>
+      <c r="CC29" s="33" t="e" vm="19">
         <f>_xlfn.IMAGE("https://flagcdn.com/w640/ae.png")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="CD29" s="38"/>
-      <c r="CE29" s="39"/>
+      <c r="CD29" s="34"/>
+      <c r="CE29" s="35"/>
     </row>
     <row r="30" spans="1:83" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="32" t="s">
+      <c r="A30" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E30" s="32" t="s">
+      <c r="E30" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F30" s="31" t="s">
+      <c r="F30" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="G30" s="32"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="32" t="s">
+      <c r="G30" s="36"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="31" t="s">
+      <c r="J30" s="36"/>
+      <c r="K30" s="36"/>
+      <c r="L30" s="36"/>
+      <c r="M30" s="36"/>
+      <c r="N30" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="O30" s="32"/>
-      <c r="P30" s="33"/>
-      <c r="Q30" s="34" t="s">
+      <c r="O30" s="36"/>
+      <c r="P30" s="41"/>
+      <c r="Q30" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="R30" s="35"/>
-      <c r="S30" s="35"/>
-      <c r="T30" s="35"/>
-      <c r="U30" s="36"/>
-      <c r="V30" s="34" t="s">
+      <c r="R30" s="43"/>
+      <c r="S30" s="43"/>
+      <c r="T30" s="43"/>
+      <c r="U30" s="44"/>
+      <c r="V30" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="W30" s="35"/>
-      <c r="X30" s="35"/>
-      <c r="Y30" s="35"/>
-      <c r="Z30" s="36"/>
-      <c r="AA30" s="31" t="s">
+      <c r="W30" s="43"/>
+      <c r="X30" s="43"/>
+      <c r="Y30" s="43"/>
+      <c r="Z30" s="44"/>
+      <c r="AA30" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="AB30" s="32"/>
-      <c r="AC30" s="33"/>
-      <c r="AD30" s="31" t="s">
+      <c r="AB30" s="36"/>
+      <c r="AC30" s="41"/>
+      <c r="AD30" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="AE30" s="32"/>
-      <c r="AF30" s="33"/>
-      <c r="AG30" s="31" t="s">
+      <c r="AE30" s="36"/>
+      <c r="AF30" s="41"/>
+      <c r="AG30" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="AH30" s="32"/>
-      <c r="AI30" s="33"/>
-      <c r="AJ30" s="32" t="s">
+      <c r="AH30" s="36"/>
+      <c r="AI30" s="41"/>
+      <c r="AJ30" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="AK30" s="32"/>
-      <c r="AL30" s="32"/>
-      <c r="AM30" s="32"/>
-      <c r="AN30" s="32"/>
-      <c r="AO30" s="31" t="s">
+      <c r="AK30" s="36"/>
+      <c r="AL30" s="36"/>
+      <c r="AM30" s="36"/>
+      <c r="AN30" s="36"/>
+      <c r="AO30" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="AP30" s="32"/>
-      <c r="AQ30" s="33"/>
-      <c r="AR30" s="31" t="s">
+      <c r="AP30" s="36"/>
+      <c r="AQ30" s="41"/>
+      <c r="AR30" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="AS30" s="32"/>
-      <c r="AT30" s="33"/>
-      <c r="AU30" s="34" t="s">
+      <c r="AS30" s="36"/>
+      <c r="AT30" s="41"/>
+      <c r="AU30" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="AV30" s="35"/>
-      <c r="AW30" s="35"/>
-      <c r="AX30" s="35"/>
-      <c r="AY30" s="36"/>
-      <c r="AZ30" s="31" t="s">
+      <c r="AV30" s="43"/>
+      <c r="AW30" s="43"/>
+      <c r="AX30" s="43"/>
+      <c r="AY30" s="44"/>
+      <c r="AZ30" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="BA30" s="32"/>
-      <c r="BB30" s="33"/>
-      <c r="BC30" s="31" t="s">
+      <c r="BA30" s="36"/>
+      <c r="BB30" s="41"/>
+      <c r="BC30" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="BD30" s="32"/>
-      <c r="BE30" s="33"/>
-      <c r="BF30" s="31" t="s">
+      <c r="BD30" s="36"/>
+      <c r="BE30" s="41"/>
+      <c r="BF30" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="BG30" s="32"/>
-      <c r="BH30" s="33"/>
-      <c r="BI30" s="34" t="s">
+      <c r="BG30" s="36"/>
+      <c r="BH30" s="41"/>
+      <c r="BI30" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="BJ30" s="35"/>
-      <c r="BK30" s="35"/>
-      <c r="BL30" s="35"/>
-      <c r="BM30" s="36"/>
-      <c r="BN30" s="31" t="s">
+      <c r="BJ30" s="43"/>
+      <c r="BK30" s="43"/>
+      <c r="BL30" s="43"/>
+      <c r="BM30" s="44"/>
+      <c r="BN30" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="BO30" s="32"/>
-      <c r="BP30" s="33"/>
-      <c r="BQ30" s="31" t="s">
+      <c r="BO30" s="36"/>
+      <c r="BP30" s="41"/>
+      <c r="BQ30" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="BR30" s="32"/>
-      <c r="BS30" s="33"/>
-      <c r="BT30" s="31" t="s">
+      <c r="BR30" s="36"/>
+      <c r="BS30" s="41"/>
+      <c r="BT30" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="BU30" s="32"/>
-      <c r="BV30" s="33"/>
-      <c r="BW30" s="31" t="s">
+      <c r="BU30" s="36"/>
+      <c r="BV30" s="41"/>
+      <c r="BW30" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="BX30" s="32"/>
-      <c r="BY30" s="33"/>
-      <c r="BZ30" s="31" t="s">
+      <c r="BX30" s="36"/>
+      <c r="BY30" s="41"/>
+      <c r="BZ30" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="CA30" s="32"/>
-      <c r="CB30" s="33"/>
-      <c r="CC30" s="31" t="s">
+      <c r="CA30" s="36"/>
+      <c r="CB30" s="41"/>
+      <c r="CC30" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="CD30" s="32"/>
-      <c r="CE30" s="33"/>
+      <c r="CD30" s="36"/>
+      <c r="CE30" s="41"/>
     </row>
     <row r="31" spans="1:83" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
+      <c r="A31" s="36"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="22" t="s">
         <v>26</v>
       </c>
@@ -11495,16 +11498,16 @@
         <v>7</v>
       </c>
       <c r="B38" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C38" s="12" t="str">
-        <v>Kimi Antonelli</v>
+        <v>Sergio Perez</v>
       </c>
       <c r="D38" s="4" t="str">
-        <v>Mercedes</v>
+        <v>Cadillac</v>
       </c>
       <c r="E38" s="2">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="F38" s="21">
         <v>0</v>
@@ -11555,7 +11558,7 @@
         <v>0</v>
       </c>
       <c r="V38" s="28">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="W38" s="23">
         <v>0</v>
@@ -11567,7 +11570,7 @@
         <v>0</v>
       </c>
       <c r="Z38" s="24">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="AA38" s="28">
         <v>0</v>
@@ -11746,13 +11749,13 @@
         <v>8</v>
       </c>
       <c r="B39" s="4">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C39" s="12" t="str">
-        <v>Nico Hulkenberg</v>
+        <v>Kimi Antonelli</v>
       </c>
       <c r="D39" s="4" t="str">
-        <v>Audi</v>
+        <v>Mercedes</v>
       </c>
       <c r="E39" s="2">
         <v>0.96</v>
@@ -11997,13 +12000,13 @@
         <v>9</v>
       </c>
       <c r="B40" s="5">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C40" s="12" t="str">
-        <v>Sergio Perez</v>
+        <v>Nico Hulkenberg</v>
       </c>
       <c r="D40" s="5" t="str">
-        <v>Cadillac</v>
+        <v>Audi</v>
       </c>
       <c r="E40" s="2">
         <v>0.96</v>
@@ -12499,16 +12502,16 @@
         <v>11</v>
       </c>
       <c r="B42" s="6">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C42" s="12" t="str">
-        <v>Isack Hadjar</v>
+        <v>Arvid Lindblad</v>
       </c>
       <c r="D42" s="6" t="str">
-        <v>Red Bull</v>
+        <v>Racing Bulls</v>
       </c>
       <c r="E42" s="2">
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="F42" s="21">
         <v>0</v>
@@ -12559,7 +12562,7 @@
         <v>0</v>
       </c>
       <c r="V42" s="28">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
       <c r="W42" s="23">
         <v>0</v>
@@ -12571,7 +12574,7 @@
         <v>0</v>
       </c>
       <c r="Z42" s="24">
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="AA42" s="28">
         <v>0</v>
@@ -12750,13 +12753,13 @@
         <v>12</v>
       </c>
       <c r="B43" s="6">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="C43" s="12" t="str">
-        <v>Arvid Lindblad</v>
+        <v>Gabriel Bortoleto</v>
       </c>
       <c r="D43" s="6" t="str">
-        <v>Racing Bulls</v>
+        <v>Audi</v>
       </c>
       <c r="E43" s="2">
         <v>0.89999999999999991</v>
@@ -13252,16 +13255,16 @@
         <v>14</v>
       </c>
       <c r="B45" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C45" s="12" t="str">
-        <v>Gabriel Bortoleto</v>
+        <v>Isack Hadjar</v>
       </c>
       <c r="D45" s="7" t="str">
-        <v>Audi</v>
+        <v>Red Bull</v>
       </c>
       <c r="E45" s="2">
-        <v>0.89400000000000002</v>
+        <v>0.87</v>
       </c>
       <c r="F45" s="21">
         <v>0</v>
@@ -13312,7 +13315,7 @@
         <v>0</v>
       </c>
       <c r="V45" s="28">
-        <v>7.45</v>
+        <v>7.25</v>
       </c>
       <c r="W45" s="23">
         <v>0</v>
@@ -13324,7 +13327,7 @@
         <v>0</v>
       </c>
       <c r="Z45" s="24">
-        <v>0.89400000000000002</v>
+        <v>0.87</v>
       </c>
       <c r="AA45" s="28">
         <v>0</v>
@@ -13503,13 +13506,13 @@
         <v>15</v>
       </c>
       <c r="B46" s="8">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C46" s="12" t="str">
-        <v>Liam Lawson</v>
+        <v>Esteban Ocon</v>
       </c>
       <c r="D46" s="8" t="str">
-        <v>Racing Bulls</v>
+        <v>Hass</v>
       </c>
       <c r="E46" s="2">
         <v>0.84</v>
@@ -13754,16 +13757,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="8">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C47" s="12" t="str">
-        <v>Esteban Ocon</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D47" s="8" t="str">
-        <v>Hass</v>
+        <v>Ferrari</v>
       </c>
       <c r="E47" s="2">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="F47" s="21">
         <v>0</v>
@@ -13814,7 +13817,7 @@
         <v>0</v>
       </c>
       <c r="V47" s="28">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W47" s="23">
         <v>0</v>
@@ -13826,7 +13829,7 @@
         <v>0</v>
       </c>
       <c r="Z47" s="24">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="AA47" s="28">
         <v>0</v>
@@ -14005,16 +14008,16 @@
         <v>17</v>
       </c>
       <c r="B48" s="9">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="C48" s="12" t="str">
-        <v>Alexander Albon</v>
+        <v>Oliver Bearman</v>
       </c>
       <c r="D48" s="9" t="str">
-        <v>Williams</v>
+        <v>Hass</v>
       </c>
       <c r="E48" s="2">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="F48" s="21">
         <v>0</v>
@@ -14065,7 +14068,7 @@
         <v>0</v>
       </c>
       <c r="V48" s="28">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W48" s="23">
         <v>0</v>
@@ -14077,7 +14080,7 @@
         <v>0</v>
       </c>
       <c r="Z48" s="24">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="AA48" s="28">
         <v>0</v>
@@ -14256,16 +14259,16 @@
         <v>18</v>
       </c>
       <c r="B49" s="9">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="C49" s="12" t="str">
-        <v>Oliver Bearman</v>
+        <v>Lance Stroll</v>
       </c>
       <c r="D49" s="9" t="str">
-        <v>Hass</v>
+        <v>Aston Martin</v>
       </c>
       <c r="E49" s="2">
-        <v>0.78</v>
+        <v>0.6</v>
       </c>
       <c r="F49" s="21">
         <v>0</v>
@@ -14316,7 +14319,7 @@
         <v>0</v>
       </c>
       <c r="V49" s="28">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="W49" s="23">
         <v>0</v>
@@ -14328,7 +14331,7 @@
         <v>0</v>
       </c>
       <c r="Z49" s="24">
-        <v>0.78</v>
+        <v>0.6</v>
       </c>
       <c r="AA49" s="28">
         <v>0</v>
@@ -14507,16 +14510,16 @@
         <v>19</v>
       </c>
       <c r="B50" s="10">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C50" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Pierre Gasly</v>
       </c>
       <c r="D50" s="10" t="str">
-        <v>Ferrari</v>
+        <v>Alpine</v>
       </c>
       <c r="E50" s="2">
-        <v>0.72</v>
+        <v>0.42</v>
       </c>
       <c r="F50" s="21">
         <v>0</v>
@@ -14567,7 +14570,7 @@
         <v>0</v>
       </c>
       <c r="V50" s="28">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="W50" s="23">
         <v>0</v>
@@ -14579,7 +14582,7 @@
         <v>0</v>
       </c>
       <c r="Z50" s="24">
-        <v>0.72</v>
+        <v>0.42</v>
       </c>
       <c r="AA50" s="28">
         <v>0</v>
@@ -14758,16 +14761,16 @@
         <v>20</v>
       </c>
       <c r="B51" s="10">
-        <v>18</v>
+        <v>77</v>
       </c>
       <c r="C51" s="12" t="str">
-        <v>Lance Stroll</v>
+        <v>Valtteri Bottas</v>
       </c>
       <c r="D51" s="10" t="str">
-        <v>Aston Martin</v>
+        <v>Cadillac</v>
       </c>
       <c r="E51" s="2">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="F51" s="21">
         <v>0</v>
@@ -14818,7 +14821,7 @@
         <v>0</v>
       </c>
       <c r="V51" s="28">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="W51" s="23">
         <v>0</v>
@@ -14830,7 +14833,7 @@
         <v>0</v>
       </c>
       <c r="Z51" s="24">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="AA51" s="28">
         <v>0</v>
@@ -15009,16 +15012,16 @@
         <v>21</v>
       </c>
       <c r="B52" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C52" s="12" t="str">
-        <v>Pierre Gasly</v>
+        <v>Liam Lawson</v>
       </c>
       <c r="D52" s="11" t="str">
-        <v>Alpine</v>
+        <v>Racing Bulls</v>
       </c>
       <c r="E52" s="2">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="F52" s="21">
         <v>0</v>
@@ -15068,8 +15071,8 @@
       <c r="U52" s="24">
         <v>0</v>
       </c>
-      <c r="V52" s="28">
-        <v>3.5</v>
+      <c r="V52" s="28" t="str">
+        <v>-</v>
       </c>
       <c r="W52" s="23">
         <v>0</v>
@@ -15081,7 +15084,7 @@
         <v>0</v>
       </c>
       <c r="Z52" s="24">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="AA52" s="28">
         <v>0</v>
@@ -15260,16 +15263,16 @@
         <v>22</v>
       </c>
       <c r="B53" s="11">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="C53" s="12" t="str">
-        <v>Valtteri Bottas</v>
+        <v>Alexander Albon</v>
       </c>
       <c r="D53" s="11" t="str">
-        <v>Cadillac</v>
+        <v>Williams</v>
       </c>
       <c r="E53" s="2">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="F53" s="21">
         <v>0</v>
@@ -15319,8 +15322,8 @@
       <c r="U53" s="24">
         <v>0</v>
       </c>
-      <c r="V53" s="28">
-        <v>1</v>
+      <c r="V53" s="28" t="str">
+        <v>-</v>
       </c>
       <c r="W53" s="23">
         <v>0</v>
@@ -15332,7 +15335,7 @@
         <v>0</v>
       </c>
       <c r="Z53" s="24">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="AA53" s="28">
         <v>0</v>
@@ -15532,33 +15535,62 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="Q3:U3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="N29:P29"/>
-    <mergeCell ref="Q29:U29"/>
-    <mergeCell ref="V29:Z29"/>
-    <mergeCell ref="V4:Z4"/>
-    <mergeCell ref="AG3:AI3"/>
-    <mergeCell ref="AJ3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="AA4:AC4"/>
-    <mergeCell ref="AD4:AF4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="AJ4:AN4"/>
-    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:M30"/>
+    <mergeCell ref="N30:P30"/>
+    <mergeCell ref="BW30:BY30"/>
+    <mergeCell ref="BZ30:CB30"/>
+    <mergeCell ref="Q30:U30"/>
+    <mergeCell ref="V30:Z30"/>
+    <mergeCell ref="AA30:AC30"/>
+    <mergeCell ref="AD30:AF30"/>
+    <mergeCell ref="AG30:AI30"/>
+    <mergeCell ref="AJ30:AN30"/>
+    <mergeCell ref="AO30:AQ30"/>
+    <mergeCell ref="AR30:AT30"/>
+    <mergeCell ref="AU30:AY30"/>
+    <mergeCell ref="CC30:CE30"/>
+    <mergeCell ref="AZ30:BB30"/>
+    <mergeCell ref="BC30:BE30"/>
+    <mergeCell ref="BF30:BH30"/>
+    <mergeCell ref="BI30:BM30"/>
+    <mergeCell ref="BN30:BP30"/>
+    <mergeCell ref="BQ30:BS30"/>
+    <mergeCell ref="BT30:BV30"/>
+    <mergeCell ref="BW29:BY29"/>
+    <mergeCell ref="BZ29:CB29"/>
+    <mergeCell ref="CC29:CE29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="AU29:AY29"/>
+    <mergeCell ref="AZ29:BB29"/>
+    <mergeCell ref="BC29:BE29"/>
+    <mergeCell ref="BF29:BH29"/>
+    <mergeCell ref="BI29:BM29"/>
+    <mergeCell ref="BN29:BP29"/>
+    <mergeCell ref="AA29:AC29"/>
+    <mergeCell ref="AD29:AF29"/>
+    <mergeCell ref="BQ29:BS29"/>
+    <mergeCell ref="BT29:BV29"/>
+    <mergeCell ref="AG29:AI29"/>
+    <mergeCell ref="AJ29:AN29"/>
+    <mergeCell ref="AO29:AQ29"/>
+    <mergeCell ref="AR29:AT29"/>
+    <mergeCell ref="CC4:CE4"/>
+    <mergeCell ref="AR4:AT4"/>
+    <mergeCell ref="AU4:AY4"/>
+    <mergeCell ref="AZ4:BB4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="BF4:BH4"/>
+    <mergeCell ref="BI4:BM4"/>
+    <mergeCell ref="BN4:BP4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BT4:BV4"/>
+    <mergeCell ref="BW4:BY4"/>
+    <mergeCell ref="BZ4:CB4"/>
     <mergeCell ref="BW3:BY3"/>
     <mergeCell ref="BZ3:CB3"/>
     <mergeCell ref="CC3:CE3"/>
@@ -15575,62 +15607,33 @@
     <mergeCell ref="BI3:BM3"/>
     <mergeCell ref="BN3:BP3"/>
     <mergeCell ref="BQ3:BS3"/>
-    <mergeCell ref="CC4:CE4"/>
-    <mergeCell ref="AR4:AT4"/>
-    <mergeCell ref="AU4:AY4"/>
-    <mergeCell ref="AZ4:BB4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="BF4:BH4"/>
-    <mergeCell ref="BI4:BM4"/>
-    <mergeCell ref="BN4:BP4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BT4:BV4"/>
-    <mergeCell ref="BW4:BY4"/>
-    <mergeCell ref="BZ4:CB4"/>
-    <mergeCell ref="BQ29:BS29"/>
-    <mergeCell ref="BT29:BV29"/>
-    <mergeCell ref="AG29:AI29"/>
-    <mergeCell ref="AJ29:AN29"/>
-    <mergeCell ref="AO29:AQ29"/>
-    <mergeCell ref="AR29:AT29"/>
-    <mergeCell ref="BW29:BY29"/>
-    <mergeCell ref="BZ29:CB29"/>
-    <mergeCell ref="CC29:CE29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="AU29:AY29"/>
-    <mergeCell ref="AZ29:BB29"/>
-    <mergeCell ref="BC29:BE29"/>
-    <mergeCell ref="BF29:BH29"/>
-    <mergeCell ref="BI29:BM29"/>
-    <mergeCell ref="BN29:BP29"/>
-    <mergeCell ref="AA29:AC29"/>
-    <mergeCell ref="AD29:AF29"/>
-    <mergeCell ref="CC30:CE30"/>
-    <mergeCell ref="AZ30:BB30"/>
-    <mergeCell ref="BC30:BE30"/>
-    <mergeCell ref="BF30:BH30"/>
-    <mergeCell ref="BI30:BM30"/>
-    <mergeCell ref="BN30:BP30"/>
-    <mergeCell ref="BQ30:BS30"/>
-    <mergeCell ref="BT30:BV30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="I30:M30"/>
-    <mergeCell ref="N30:P30"/>
-    <mergeCell ref="BW30:BY30"/>
-    <mergeCell ref="BZ30:CB30"/>
-    <mergeCell ref="Q30:U30"/>
-    <mergeCell ref="V30:Z30"/>
-    <mergeCell ref="AA30:AC30"/>
-    <mergeCell ref="AD30:AF30"/>
-    <mergeCell ref="AG30:AI30"/>
-    <mergeCell ref="AJ30:AN30"/>
-    <mergeCell ref="AO30:AQ30"/>
-    <mergeCell ref="AR30:AT30"/>
-    <mergeCell ref="AU30:AY30"/>
+    <mergeCell ref="V4:Z4"/>
+    <mergeCell ref="AG3:AI3"/>
+    <mergeCell ref="AJ3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="AA4:AC4"/>
+    <mergeCell ref="AD4:AF4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="AJ4:AN4"/>
+    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="N29:P29"/>
+    <mergeCell ref="Q29:U29"/>
+    <mergeCell ref="V29:Z29"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="Q3:U3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="Q4:U4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B27 D6:D27 B32:B53 D32:D53">
     <cfRule type="expression" dxfId="65" priority="329">
@@ -15962,7 +15965,7 @@
       </c>
       <c r="N5" s="29">
         <f>Simplified!G8</f>
-        <v>3.0000000000000027E-2</v>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="O5" s="4">
         <v>6</v>
@@ -16047,7 +16050,7 @@
       </c>
       <c r="N7" s="29">
         <f>Simplified!G12</f>
-        <v>-5.9999999999999942E-2</v>
+        <v>-0.92999999999999994</v>
       </c>
       <c r="O7" s="6">
         <v>41</v>
@@ -16058,20 +16061,20 @@
         <v>7</v>
       </c>
       <c r="B8" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="12" t="str">
-        <v>Kimi Antonelli</v>
+        <v>Sergio Perez</v>
       </c>
       <c r="D8" s="4" t="str">
-        <v>Mercedes</v>
+        <v>Cadillac</v>
       </c>
       <c r="E8" s="2">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="G8" s="45">
         <f>K8-K9</f>
-        <v>3.0000000000000027E-2</v>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="H8" s="4">
         <v>3</v>
@@ -16091,7 +16094,7 @@
       </c>
       <c r="N8" s="29">
         <f>Simplified!G14</f>
-        <v>5.9999999999999942E-2</v>
+        <v>0.12</v>
       </c>
       <c r="O8" s="7">
         <v>87</v>
@@ -16102,13 +16105,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C9" s="12" t="str">
-        <v>Nico Hulkenberg</v>
+        <v>Kimi Antonelli</v>
       </c>
       <c r="D9" s="4" t="str">
-        <v>Audi</v>
+        <v>Mercedes</v>
       </c>
       <c r="E9" s="2">
         <v>0.96</v>
@@ -16125,14 +16128,14 @@
       </c>
       <c r="K9" s="2">
         <f>Ratings!E13</f>
-        <v>0.89999999999999991</v>
+        <v>0.87</v>
       </c>
       <c r="M9" s="8">
         <v>55</v>
       </c>
       <c r="N9" s="29">
         <f>Simplified!G16</f>
-        <v>0.18000000000000005</v>
+        <v>1.02</v>
       </c>
       <c r="O9" s="8">
         <v>23</v>
@@ -16143,13 +16146,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="5">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C10" s="12" t="str">
-        <v>Sergio Perez</v>
+        <v>Nico Hulkenberg</v>
       </c>
       <c r="D10" s="5" t="str">
-        <v>Cadillac</v>
+        <v>Audi</v>
       </c>
       <c r="E10" s="2">
         <v>0.96</v>
@@ -16176,7 +16179,7 @@
       </c>
       <c r="N10" s="29">
         <f>Simplified!G18</f>
-        <v>6.5999999999999948E-2</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="O10" s="9">
         <v>5</v>
@@ -16217,7 +16220,7 @@
       </c>
       <c r="N11" s="29">
         <f>Simplified!G20</f>
-        <v>0.84</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="O11" s="10">
         <v>77</v>
@@ -16228,20 +16231,20 @@
         <v>11</v>
       </c>
       <c r="B12" s="6">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C12" s="12" t="str">
-        <v>Isack Hadjar</v>
+        <v>Arvid Lindblad</v>
       </c>
       <c r="D12" s="6" t="str">
-        <v>Red Bull</v>
+        <v>Racing Bulls</v>
       </c>
       <c r="E12" s="2">
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="G12" s="45">
         <f>K12-K13</f>
-        <v>-5.9999999999999942E-2</v>
+        <v>-0.92999999999999994</v>
       </c>
       <c r="H12" s="6">
         <v>30</v>
@@ -16254,7 +16257,7 @@
       </c>
       <c r="K12" s="2">
         <f>Ratings!E16</f>
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="M12" s="11">
         <v>14</v>
@@ -16272,13 +16275,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="C13" s="12" t="str">
-        <v>Arvid Lindblad</v>
+        <v>Gabriel Bortoleto</v>
       </c>
       <c r="D13" s="6" t="str">
-        <v>Racing Bulls</v>
+        <v>Audi</v>
       </c>
       <c r="E13" s="2">
         <v>0.89999999999999991</v>
@@ -16295,7 +16298,7 @@
       </c>
       <c r="K13" s="2">
         <f>Ratings!E17</f>
-        <v>0.89999999999999991</v>
+        <v>0.92999999999999994</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
@@ -16316,7 +16319,7 @@
       </c>
       <c r="G14" s="45">
         <f>K14-K15</f>
-        <v>5.9999999999999942E-2</v>
+        <v>0.12</v>
       </c>
       <c r="H14" s="7">
         <v>31</v>
@@ -16337,16 +16340,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="12" t="str">
-        <v>Gabriel Bortoleto</v>
+        <v>Isack Hadjar</v>
       </c>
       <c r="D15" s="7" t="str">
-        <v>Audi</v>
+        <v>Red Bull</v>
       </c>
       <c r="E15" s="2">
-        <v>0.89400000000000002</v>
+        <v>0.87</v>
       </c>
       <c r="G15" s="45"/>
       <c r="H15" s="7">
@@ -16360,7 +16363,7 @@
       </c>
       <c r="K15" s="2">
         <f>Ratings!E19</f>
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
@@ -16368,20 +16371,20 @@
         <v>15</v>
       </c>
       <c r="B16" s="8">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C16" s="12" t="str">
-        <v>Liam Lawson</v>
+        <v>Esteban Ocon</v>
       </c>
       <c r="D16" s="8" t="str">
-        <v>Racing Bulls</v>
+        <v>Hass</v>
       </c>
       <c r="E16" s="2">
         <v>0.84</v>
       </c>
       <c r="G16" s="45">
         <f>K16-K17</f>
-        <v>0.18000000000000005</v>
+        <v>1.02</v>
       </c>
       <c r="H16" s="8">
         <v>55</v>
@@ -16402,16 +16405,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="8">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C17" s="12" t="str">
-        <v>Esteban Ocon</v>
+        <v>Charles Leclerc</v>
       </c>
       <c r="D17" s="8" t="str">
-        <v>Hass</v>
+        <v>Ferrari</v>
       </c>
       <c r="E17" s="2">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="G17" s="45"/>
       <c r="H17" s="8">
@@ -16425,7 +16428,7 @@
       </c>
       <c r="K17" s="2">
         <f>Ratings!E21</f>
-        <v>0.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -16433,20 +16436,20 @@
         <v>17</v>
       </c>
       <c r="B18" s="9">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="C18" s="12" t="str">
-        <v>Alexander Albon</v>
+        <v>Oliver Bearman</v>
       </c>
       <c r="D18" s="9" t="str">
-        <v>Williams</v>
+        <v>Hass</v>
       </c>
       <c r="E18" s="2">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="G18" s="45">
         <f>K18-K19</f>
-        <v>6.5999999999999948E-2</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="H18" s="9">
         <v>27</v>
@@ -16467,16 +16470,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="9">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="C19" s="12" t="str">
-        <v>Oliver Bearman</v>
+        <v>Lance Stroll</v>
       </c>
       <c r="D19" s="9" t="str">
-        <v>Hass</v>
+        <v>Aston Martin</v>
       </c>
       <c r="E19" s="2">
-        <v>0.78</v>
+        <v>0.6</v>
       </c>
       <c r="G19" s="45"/>
       <c r="H19" s="9">
@@ -16490,7 +16493,7 @@
       </c>
       <c r="K19" s="2">
         <f>Ratings!E23</f>
-        <v>0.89400000000000002</v>
+        <v>0.89999999999999991</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
@@ -16498,20 +16501,20 @@
         <v>19</v>
       </c>
       <c r="B20" s="10">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C20" s="12" t="str">
-        <v>Charles Leclerc</v>
+        <v>Pierre Gasly</v>
       </c>
       <c r="D20" s="10" t="str">
-        <v>Ferrari</v>
+        <v>Alpine</v>
       </c>
       <c r="E20" s="2">
-        <v>0.72</v>
+        <v>0.42</v>
       </c>
       <c r="G20" s="45">
         <f>K20-K21</f>
-        <v>0.84</v>
+        <v>0.92999999999999994</v>
       </c>
       <c r="H20" s="10">
         <v>11</v>
@@ -16524,7 +16527,7 @@
       </c>
       <c r="K20" s="2">
         <f>Ratings!E24</f>
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
@@ -16532,16 +16535,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="10">
-        <v>18</v>
+        <v>77</v>
       </c>
       <c r="C21" s="12" t="str">
-        <v>Lance Stroll</v>
+        <v>Valtteri Bottas</v>
       </c>
       <c r="D21" s="10" t="str">
-        <v>Aston Martin</v>
+        <v>Cadillac</v>
       </c>
       <c r="E21" s="2">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="G21" s="45"/>
       <c r="H21" s="10">
@@ -16555,7 +16558,7 @@
       </c>
       <c r="K21" s="2">
         <f>Ratings!E25</f>
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
@@ -16563,16 +16566,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C22" s="12" t="str">
-        <v>Pierre Gasly</v>
+        <v>Liam Lawson</v>
       </c>
       <c r="D22" s="11" t="str">
-        <v>Alpine</v>
+        <v>Racing Bulls</v>
       </c>
       <c r="E22" s="2">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="G22" s="45">
         <f>K22-K23</f>
@@ -16597,16 +16600,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="11">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="C23" s="12" t="str">
-        <v>Valtteri Bottas</v>
+        <v>Alexander Albon</v>
       </c>
       <c r="D23" s="11" t="str">
-        <v>Cadillac</v>
+        <v>Williams</v>
       </c>
       <c r="E23" s="2">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="G23" s="45"/>
       <c r="H23" s="11">
@@ -16684,7 +16687,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4 G2 G6 G8 G10 G12 G14 G16 G18 G20 G22">
+  <conditionalFormatting sqref="G2 G4 G6 G8 G10 G12 G14 G16 G18 G20 G22">
     <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="percentile" val="0"/>

</xml_diff>